<commit_message>
feat(students): update student form pages, dossier export, attendance, guest book, and fix table layout
</commit_message>
<xml_diff>
--- a/public/DATABASE MURID SMP 2026-2027.xlsx
+++ b/public/DATABASE MURID SMP 2026-2027.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23901"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\SMP ANAK SALEH\ADMIN - TU\TA'ARUF\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\IHWAN\Project\sans-smp\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96DE8275-6142-4CEC-A98B-C9A552E4076D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42B3B393-A9F0-42AD-ADAA-6B11D3B6EF80}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,22 +20,11 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">MASTER!$A$1:$DH$14</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2696" uniqueCount="1040">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2694" uniqueCount="1039">
   <si>
     <t>Timestamp</t>
   </si>
@@ -2806,9 +2795,6 @@
   </si>
   <si>
     <t>linda.a.rowman@gmail.com</t>
-  </si>
-  <si>
-    <t>Jl. Mt Haryono 9 No.326, Dinoyo, Kec. Lowokwaru, Kota Malang. 65145</t>
   </si>
   <si>
     <t>Ir. RAHMAN ARIFUDDIN, S.T., M.T</t>
@@ -3302,8 +3288,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+  <cellXfs count="38">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -3322,7 +3308,7 @@
     <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -3331,28 +3317,25 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
@@ -3364,13 +3347,13 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -3379,40 +3362,40 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" quotePrefix="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="6" fillId="4" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -3849,7 +3832,7 @@
     <col min="4" max="4" width="28.85546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="81" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10" style="10" customWidth="1"/>
-    <col min="7" max="7" width="15.85546875" style="13" customWidth="1"/>
+    <col min="7" max="7" width="15.85546875" style="12" customWidth="1"/>
     <col min="8" max="9" width="24.28515625" style="10" customWidth="1"/>
     <col min="10" max="10" width="26.85546875" style="10" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="38.28515625" bestFit="1" customWidth="1"/>
@@ -3857,7 +3840,7 @@
     <col min="13" max="13" width="17.85546875" style="10" bestFit="1" customWidth="1"/>
     <col min="14" max="15" width="18.28515625" style="10" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="15.28515625" style="10" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="17.28515625" style="13" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="17.28515625" style="12" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="20.85546875" style="10" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="22.28515625" style="10" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="31" bestFit="1" customWidth="1"/>
@@ -3907,7 +3890,7 @@
     <col min="64" max="64" width="33.140625" bestFit="1" customWidth="1"/>
     <col min="65" max="65" width="90.85546875" bestFit="1" customWidth="1"/>
     <col min="66" max="66" width="38.28515625" style="10" bestFit="1" customWidth="1"/>
-    <col min="67" max="67" width="31.7109375" style="22" bestFit="1" customWidth="1"/>
+    <col min="67" max="67" width="31.7109375" style="21" bestFit="1" customWidth="1"/>
     <col min="68" max="68" width="29.42578125" bestFit="1" customWidth="1"/>
     <col min="69" max="69" width="60.28515625" bestFit="1" customWidth="1"/>
     <col min="70" max="70" width="48.85546875" bestFit="1" customWidth="1"/>
@@ -3978,7 +3961,7 @@
         <v>744</v>
       </c>
       <c r="H1" s="8" t="s">
-        <v>1029</v>
+        <v>1028</v>
       </c>
       <c r="I1" s="8" t="s">
         <v>798</v>
@@ -4152,7 +4135,7 @@
       <c r="BN1" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="BO1" s="20" t="s">
+      <c r="BO1" s="19" t="s">
         <v>55</v>
       </c>
       <c r="BP1" s="9" t="s">
@@ -4292,10 +4275,10 @@
       </c>
     </row>
     <row r="2" spans="1:113" s="7" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="13">
+      <c r="A2" s="12">
         <v>1</v>
       </c>
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="14" t="s">
         <v>831</v>
       </c>
       <c r="C2" s="7" t="s">
@@ -4305,48 +4288,48 @@
         <v>598</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>940</v>
-      </c>
-      <c r="F2" s="19" t="s">
-        <v>924</v>
-      </c>
-      <c r="G2" s="14" t="s">
+        <v>939</v>
+      </c>
+      <c r="F2" s="18" t="s">
+        <v>923</v>
+      </c>
+      <c r="G2" s="13" t="s">
         <v>815</v>
       </c>
-      <c r="H2" s="37" t="s">
-        <v>1036</v>
-      </c>
-      <c r="I2" s="14" t="s">
-        <v>937</v>
-      </c>
-      <c r="J2" s="13" t="s">
+      <c r="H2" s="36" t="s">
+        <v>1035</v>
+      </c>
+      <c r="I2" s="13" t="s">
+        <v>936</v>
+      </c>
+      <c r="J2" s="12" t="s">
         <v>575</v>
       </c>
       <c r="K2" s="7" t="s">
         <v>572</v>
       </c>
-      <c r="L2" s="13">
+      <c r="L2" s="12">
         <v>7</v>
       </c>
-      <c r="M2" s="13" t="s">
+      <c r="M2" s="12" t="s">
         <v>801</v>
       </c>
-      <c r="N2" s="13" t="s">
+      <c r="N2" s="12" t="s">
         <v>573</v>
       </c>
-      <c r="O2" s="13" t="s">
+      <c r="O2" s="12" t="s">
         <v>574</v>
       </c>
-      <c r="P2" s="13" t="s">
+      <c r="P2" s="12" t="s">
         <v>286</v>
       </c>
-      <c r="Q2" s="13" t="s">
+      <c r="Q2" s="12" t="s">
         <v>226</v>
       </c>
-      <c r="R2" s="23" t="s">
+      <c r="R2" s="22" t="s">
         <v>765</v>
       </c>
-      <c r="S2" s="17" t="e">
+      <c r="S2" s="16" t="e">
         <f ca="1">DATEDIF(R2, TODAY(), "Y") &amp; " Tahun " &amp; DATEDIF(R2, TODAY(), "YM") &amp; " Bulan " &amp; DATEDIF(R2, TODAY(), "MD") &amp; " Hari"</f>
         <v>#VALUE!</v>
       </c>
@@ -4356,10 +4339,10 @@
       <c r="V2" s="7" t="s">
         <v>576</v>
       </c>
-      <c r="W2" s="13" t="s">
+      <c r="W2" s="12" t="s">
         <v>577</v>
       </c>
-      <c r="X2" s="13" t="s">
+      <c r="X2" s="12" t="s">
         <v>577</v>
       </c>
       <c r="Y2" s="7" t="s">
@@ -4371,7 +4354,7 @@
       <c r="AA2" s="7" t="s">
         <v>490</v>
       </c>
-      <c r="AB2" s="13">
+      <c r="AB2" s="12">
         <v>65145</v>
       </c>
       <c r="AC2" s="7" t="s">
@@ -4410,13 +4393,13 @@
       <c r="AN2" s="7" t="s">
         <v>236</v>
       </c>
-      <c r="AO2" s="13">
+      <c r="AO2" s="12">
         <v>41</v>
       </c>
-      <c r="AP2" s="13">
+      <c r="AP2" s="12">
         <v>155</v>
       </c>
-      <c r="AQ2" s="13" t="s">
+      <c r="AQ2" s="12" t="s">
         <v>238</v>
       </c>
       <c r="AR2" s="7" t="s">
@@ -4434,8 +4417,8 @@
       <c r="AV2" s="7" t="s">
         <v>226</v>
       </c>
-      <c r="AW2" s="15" t="s">
-        <v>938</v>
+      <c r="AW2" s="14" t="s">
+        <v>937</v>
       </c>
       <c r="AX2" s="7" t="s">
         <v>584</v>
@@ -4443,10 +4426,10 @@
       <c r="AY2" s="7" t="s">
         <v>585</v>
       </c>
-      <c r="BA2" s="13" t="s">
+      <c r="BA2" s="12" t="s">
         <v>577</v>
       </c>
-      <c r="BB2" s="13" t="s">
+      <c r="BB2" s="12" t="s">
         <v>577</v>
       </c>
       <c r="BC2" s="7" t="s">
@@ -4458,16 +4441,16 @@
       <c r="BE2" s="7" t="s">
         <v>490</v>
       </c>
-      <c r="BF2" s="13">
+      <c r="BF2" s="12">
         <v>65145</v>
       </c>
       <c r="BG2" s="7" t="s">
         <v>161</v>
       </c>
-      <c r="BH2" s="13" t="s">
+      <c r="BH2" s="12" t="s">
         <v>162</v>
       </c>
-      <c r="BI2" s="13" t="s">
+      <c r="BI2" s="12" t="s">
         <v>586</v>
       </c>
       <c r="BJ2" s="7" t="s">
@@ -4483,10 +4466,10 @@
       <c r="BM2" s="7" t="s">
         <v>870</v>
       </c>
-      <c r="BN2" s="13">
+      <c r="BN2" s="12">
         <v>1500056</v>
       </c>
-      <c r="BO2" s="21" t="s">
+      <c r="BO2" s="20" t="s">
         <v>257</v>
       </c>
       <c r="BP2" s="7" t="s">
@@ -4501,8 +4484,8 @@
       <c r="BS2" s="7" t="s">
         <v>593</v>
       </c>
-      <c r="BT2" s="15" t="s">
-        <v>939</v>
+      <c r="BT2" s="14" t="s">
+        <v>938</v>
       </c>
       <c r="BU2" s="7" t="s">
         <v>594</v>
@@ -4510,10 +4493,10 @@
       <c r="BV2" s="7" t="s">
         <v>576</v>
       </c>
-      <c r="BW2" s="13" t="s">
+      <c r="BW2" s="12" t="s">
         <v>577</v>
       </c>
-      <c r="BX2" s="13" t="s">
+      <c r="BX2" s="12" t="s">
         <v>577</v>
       </c>
       <c r="BY2" s="7" t="s">
@@ -4525,7 +4508,7 @@
       <c r="CA2" s="7" t="s">
         <v>490</v>
       </c>
-      <c r="CB2" s="13">
+      <c r="CB2" s="12">
         <v>65145</v>
       </c>
       <c r="CC2" s="7" t="s">
@@ -4534,7 +4517,7 @@
       <c r="CD2" s="7" t="s">
         <v>162</v>
       </c>
-      <c r="CE2" s="13" t="s">
+      <c r="CE2" s="12" t="s">
         <v>579</v>
       </c>
       <c r="CF2" s="7" t="s">
@@ -4549,7 +4532,7 @@
       <c r="CI2" s="7" t="s">
         <v>897</v>
       </c>
-      <c r="CJ2" s="13" t="s">
+      <c r="CJ2" s="12" t="s">
         <v>597</v>
       </c>
       <c r="CK2" s="7" t="s">
@@ -4564,13 +4547,13 @@
       <c r="CN2" s="7" t="s">
         <v>841</v>
       </c>
-      <c r="CP2" s="13"/>
+      <c r="CP2" s="12"/>
     </row>
     <row r="3" spans="1:113" s="7" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="13">
+      <c r="A3" s="12">
         <v>2</v>
       </c>
-      <c r="B3" s="15" t="s">
+      <c r="B3" s="14" t="s">
         <v>832</v>
       </c>
       <c r="C3" s="7" t="s">
@@ -4582,46 +4565,46 @@
       <c r="E3" s="7" t="s">
         <v>803</v>
       </c>
-      <c r="F3" s="14" t="s">
-        <v>925</v>
-      </c>
-      <c r="G3" s="14" t="s">
+      <c r="F3" s="13" t="s">
+        <v>924</v>
+      </c>
+      <c r="G3" s="13" t="s">
         <v>809</v>
       </c>
-      <c r="H3" s="15"/>
-      <c r="I3" s="14" t="s">
-        <v>941</v>
-      </c>
-      <c r="J3" s="14" t="s">
-        <v>1005</v>
+      <c r="H3" s="14"/>
+      <c r="I3" s="13" t="s">
+        <v>940</v>
+      </c>
+      <c r="J3" s="13" t="s">
+        <v>1004</v>
       </c>
       <c r="K3" s="7" t="s">
         <v>750</v>
       </c>
-      <c r="L3" s="13">
+      <c r="L3" s="12">
         <v>7</v>
       </c>
-      <c r="M3" s="13" t="s">
+      <c r="M3" s="12" t="s">
         <v>801</v>
       </c>
-      <c r="N3" s="13" t="s">
+      <c r="N3" s="12" t="s">
         <v>756</v>
       </c>
-      <c r="O3" s="13" t="s">
+      <c r="O3" s="12" t="s">
         <v>657</v>
       </c>
-      <c r="P3" s="13" t="s">
+      <c r="P3" s="12" t="s">
         <v>149</v>
       </c>
-      <c r="Q3" s="13" t="s">
+      <c r="Q3" s="12" t="s">
         <v>226</v>
       </c>
-      <c r="R3" s="17" t="s">
+      <c r="R3" s="16" t="s">
         <v>816</v>
       </c>
-      <c r="S3" s="17" t="str">
+      <c r="S3" s="16" t="str">
         <f ca="1">DATEDIF(R3, TODAY(), "Y") &amp; " Tahun " &amp; DATEDIF(R3, TODAY(), "YM") &amp; " Bulan " &amp; DATEDIF(R3, TODAY(), "MD") &amp; " Hari"</f>
-        <v>13 Tahun 0 Bulan 13 Hari</v>
+        <v>13 Tahun 1 Bulan 6 Hari</v>
       </c>
       <c r="T3" s="7" t="s">
         <v>151</v>
@@ -4629,10 +4612,10 @@
       <c r="V3" s="7" t="s">
         <v>775</v>
       </c>
-      <c r="W3" s="13">
+      <c r="W3" s="12">
         <v>19</v>
       </c>
-      <c r="X3" s="13" t="s">
+      <c r="X3" s="12" t="s">
         <v>533</v>
       </c>
       <c r="Y3" s="7" t="s">
@@ -4644,7 +4627,7 @@
       <c r="AA3" s="7" t="s">
         <v>490</v>
       </c>
-      <c r="AB3" s="13">
+      <c r="AB3" s="12">
         <v>65152</v>
       </c>
       <c r="AC3" s="7">
@@ -4683,13 +4666,13 @@
       <c r="AN3" s="7" t="s">
         <v>294</v>
       </c>
-      <c r="AO3" s="13">
+      <c r="AO3" s="12">
         <v>41</v>
       </c>
-      <c r="AP3" s="13">
+      <c r="AP3" s="12">
         <v>158</v>
       </c>
-      <c r="AQ3" s="13" t="s">
+      <c r="AQ3" s="12" t="s">
         <v>238</v>
       </c>
       <c r="AR3" s="7" t="s">
@@ -4707,8 +4690,8 @@
       <c r="AV3" s="7" t="s">
         <v>849</v>
       </c>
-      <c r="AW3" s="15" t="s">
-        <v>942</v>
+      <c r="AW3" s="14" t="s">
+        <v>941</v>
       </c>
       <c r="AX3" s="7" t="s">
         <v>669</v>
@@ -4716,10 +4699,10 @@
       <c r="AY3" s="7" t="s">
         <v>775</v>
       </c>
-      <c r="BA3" s="13">
+      <c r="BA3" s="12">
         <v>19</v>
       </c>
-      <c r="BB3" s="13" t="s">
+      <c r="BB3" s="12" t="s">
         <v>533</v>
       </c>
       <c r="BC3" s="7" t="s">
@@ -4731,16 +4714,16 @@
       <c r="BE3" s="11" t="s">
         <v>787</v>
       </c>
-      <c r="BF3" s="13">
+      <c r="BF3" s="12">
         <v>65125</v>
       </c>
       <c r="BG3" s="7" t="s">
         <v>161</v>
       </c>
-      <c r="BH3" s="13" t="s">
+      <c r="BH3" s="12" t="s">
         <v>162</v>
       </c>
-      <c r="BI3" s="13" t="s">
+      <c r="BI3" s="12" t="s">
         <v>671</v>
       </c>
       <c r="BJ3" s="7" t="s">
@@ -4756,10 +4739,10 @@
       <c r="BM3" s="7" t="s">
         <v>871</v>
       </c>
-      <c r="BN3" s="13" t="s">
+      <c r="BN3" s="12" t="s">
         <v>676</v>
       </c>
-      <c r="BO3" s="21">
+      <c r="BO3" s="20">
         <v>10</v>
       </c>
       <c r="BP3" s="7" t="s">
@@ -4774,8 +4757,8 @@
       <c r="BS3" s="7" t="s">
         <v>711</v>
       </c>
-      <c r="BT3" s="15" t="s">
-        <v>943</v>
+      <c r="BT3" s="14" t="s">
+        <v>942</v>
       </c>
       <c r="BU3" s="7" t="s">
         <v>679</v>
@@ -4783,10 +4766,10 @@
       <c r="BV3" s="7" t="s">
         <v>775</v>
       </c>
-      <c r="BW3" s="13">
+      <c r="BW3" s="12">
         <v>19</v>
       </c>
-      <c r="BX3" s="13" t="s">
+      <c r="BX3" s="12" t="s">
         <v>533</v>
       </c>
       <c r="BY3" s="7" t="s">
@@ -4798,7 +4781,7 @@
       <c r="CA3" s="11" t="s">
         <v>787</v>
       </c>
-      <c r="CB3" s="13">
+      <c r="CB3" s="12">
         <v>651252</v>
       </c>
       <c r="CC3" s="7" t="s">
@@ -4807,7 +4790,7 @@
       <c r="CD3" s="7" t="s">
         <v>162</v>
       </c>
-      <c r="CE3" s="13" t="s">
+      <c r="CE3" s="12" t="s">
         <v>680</v>
       </c>
       <c r="CF3" s="7" t="s">
@@ -4822,7 +4805,7 @@
       <c r="CI3" s="7" t="s">
         <v>775</v>
       </c>
-      <c r="CJ3" s="19" t="s">
+      <c r="CJ3" s="18" t="s">
         <v>901</v>
       </c>
       <c r="CK3" s="7" t="s">
@@ -4840,7 +4823,7 @@
       <c r="CO3" s="11" t="s">
         <v>903</v>
       </c>
-      <c r="CP3" s="13">
+      <c r="CP3" s="12">
         <v>29708</v>
       </c>
       <c r="CQ3" s="7" t="s">
@@ -4899,10 +4882,10 @@
       </c>
     </row>
     <row r="4" spans="1:113" s="7" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="13">
+      <c r="A4" s="12">
         <v>3</v>
       </c>
-      <c r="B4" s="15" t="s">
+      <c r="B4" s="14" t="s">
         <v>831</v>
       </c>
       <c r="C4" s="7" t="s">
@@ -4912,46 +4895,46 @@
         <v>834</v>
       </c>
       <c r="E4" s="7" t="s">
+        <v>943</v>
+      </c>
+      <c r="F4" s="13" t="s">
+        <v>925</v>
+      </c>
+      <c r="G4" s="13" t="s">
+        <v>812</v>
+      </c>
+      <c r="H4" s="14"/>
+      <c r="I4" s="13" t="s">
         <v>944</v>
       </c>
-      <c r="F4" s="14" t="s">
-        <v>926</v>
-      </c>
-      <c r="G4" s="14" t="s">
-        <v>812</v>
-      </c>
-      <c r="H4" s="15"/>
-      <c r="I4" s="14" t="s">
-        <v>945</v>
-      </c>
-      <c r="J4" s="14" t="s">
-        <v>1006</v>
+      <c r="J4" s="13" t="s">
+        <v>1005</v>
       </c>
       <c r="K4" s="7" t="s">
         <v>749</v>
       </c>
-      <c r="L4" s="13">
+      <c r="L4" s="12">
         <v>7</v>
       </c>
-      <c r="M4" s="13" t="s">
+      <c r="M4" s="12" t="s">
         <v>801</v>
       </c>
-      <c r="N4" s="13" t="s">
+      <c r="N4" s="12" t="s">
         <v>755</v>
       </c>
-      <c r="O4" s="13" t="s">
+      <c r="O4" s="12" t="s">
         <v>614</v>
       </c>
-      <c r="P4" s="13" t="s">
+      <c r="P4" s="12" t="s">
         <v>149</v>
       </c>
-      <c r="Q4" s="13" t="s">
+      <c r="Q4" s="12" t="s">
         <v>226</v>
       </c>
-      <c r="R4" s="17" t="s">
+      <c r="R4" s="16" t="s">
         <v>766</v>
       </c>
-      <c r="S4" s="17" t="e">
+      <c r="S4" s="16" t="e">
         <f t="shared" ref="S4:S12" ca="1" si="1">DATEDIF(R4, TODAY(), "Y") &amp; " Tahun " &amp; DATEDIF(R4, TODAY(), "YM") &amp; " Bulan " &amp; DATEDIF(R4, TODAY(), "MD") &amp; " Hari"</f>
         <v>#VALUE!</v>
       </c>
@@ -4961,10 +4944,10 @@
       <c r="V4" s="7" t="s">
         <v>616</v>
       </c>
-      <c r="W4" s="13" t="s">
+      <c r="W4" s="12" t="s">
         <v>577</v>
       </c>
-      <c r="X4" s="13" t="s">
+      <c r="X4" s="12" t="s">
         <v>487</v>
       </c>
       <c r="Y4" s="7" t="s">
@@ -4976,7 +4959,7 @@
       <c r="AA4" s="7" t="s">
         <v>490</v>
       </c>
-      <c r="AB4" s="13">
+      <c r="AB4" s="12">
         <v>65141</v>
       </c>
       <c r="AC4" s="7" t="s">
@@ -5009,13 +4992,13 @@
       <c r="AN4" s="7" t="s">
         <v>236</v>
       </c>
-      <c r="AO4" s="13">
+      <c r="AO4" s="12">
         <v>42</v>
       </c>
-      <c r="AP4" s="13">
+      <c r="AP4" s="12">
         <v>150</v>
       </c>
-      <c r="AQ4" s="13" t="s">
+      <c r="AQ4" s="12" t="s">
         <v>164</v>
       </c>
       <c r="AR4" s="7" t="s">
@@ -5033,8 +5016,8 @@
       <c r="AV4" s="7" t="s">
         <v>226</v>
       </c>
-      <c r="AW4" s="15" t="s">
-        <v>946</v>
+      <c r="AW4" s="14" t="s">
+        <v>945</v>
       </c>
       <c r="AX4" s="7" t="s">
         <v>623</v>
@@ -5042,10 +5025,10 @@
       <c r="AY4" s="7" t="s">
         <v>624</v>
       </c>
-      <c r="BA4" s="13" t="s">
+      <c r="BA4" s="12" t="s">
         <v>577</v>
       </c>
-      <c r="BB4" s="13" t="s">
+      <c r="BB4" s="12" t="s">
         <v>487</v>
       </c>
       <c r="BC4" s="7" t="s">
@@ -5057,16 +5040,16 @@
       <c r="BE4" s="7" t="s">
         <v>490</v>
       </c>
-      <c r="BF4" s="13">
+      <c r="BF4" s="12">
         <v>65141</v>
       </c>
       <c r="BG4" s="7" t="s">
         <v>161</v>
       </c>
-      <c r="BH4" s="13" t="s">
+      <c r="BH4" s="12" t="s">
         <v>162</v>
       </c>
-      <c r="BI4" s="19" t="s">
+      <c r="BI4" s="18" t="s">
         <v>863</v>
       </c>
       <c r="BJ4" s="7" t="s">
@@ -5082,10 +5065,10 @@
       <c r="BM4" s="7" t="s">
         <v>872</v>
       </c>
-      <c r="BN4" s="13" t="s">
+      <c r="BN4" s="12" t="s">
         <v>629</v>
       </c>
-      <c r="BO4" s="21" t="s">
+      <c r="BO4" s="20" t="s">
         <v>630</v>
       </c>
       <c r="BP4" s="7" t="s">
@@ -5100,19 +5083,19 @@
       <c r="BS4" s="7" t="s">
         <v>226</v>
       </c>
-      <c r="BT4" s="15" t="s">
-        <v>947</v>
-      </c>
-      <c r="BU4" s="18" t="s">
+      <c r="BT4" s="14" t="s">
+        <v>946</v>
+      </c>
+      <c r="BU4" s="17" t="s">
         <v>888</v>
       </c>
       <c r="BV4" s="7" t="s">
         <v>633</v>
       </c>
-      <c r="BW4" s="13" t="s">
+      <c r="BW4" s="12" t="s">
         <v>577</v>
       </c>
-      <c r="BX4" s="13" t="s">
+      <c r="BX4" s="12" t="s">
         <v>487</v>
       </c>
       <c r="BY4" s="7" t="s">
@@ -5124,7 +5107,7 @@
       <c r="CA4" s="11" t="s">
         <v>490</v>
       </c>
-      <c r="CB4" s="13">
+      <c r="CB4" s="12">
         <v>65141</v>
       </c>
       <c r="CC4" s="7" t="s">
@@ -5133,7 +5116,7 @@
       <c r="CD4" s="7" t="s">
         <v>162</v>
       </c>
-      <c r="CE4" s="13" t="s">
+      <c r="CE4" s="12" t="s">
         <v>618</v>
       </c>
       <c r="CF4" s="7" t="s">
@@ -5148,7 +5131,7 @@
       <c r="CI4" s="7" t="s">
         <v>152</v>
       </c>
-      <c r="CJ4" s="13" t="s">
+      <c r="CJ4" s="12" t="s">
         <v>152</v>
       </c>
       <c r="CK4" s="7" t="s">
@@ -5163,13 +5146,13 @@
       <c r="CN4" s="7" t="s">
         <v>841</v>
       </c>
-      <c r="CP4" s="13"/>
+      <c r="CP4" s="12"/>
     </row>
     <row r="5" spans="1:113" s="7" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="13">
+      <c r="A5" s="12">
         <v>4</v>
       </c>
-      <c r="B5" s="15" t="s">
+      <c r="B5" s="14" t="s">
         <v>830</v>
       </c>
       <c r="C5" s="7" t="s">
@@ -5181,46 +5164,46 @@
       <c r="E5" s="7" t="s">
         <v>824</v>
       </c>
-      <c r="F5" s="14" t="s">
-        <v>927</v>
-      </c>
-      <c r="G5" s="14" t="s">
+      <c r="F5" s="13" t="s">
+        <v>926</v>
+      </c>
+      <c r="G5" s="13" t="s">
         <v>821</v>
       </c>
-      <c r="H5" s="37" t="s">
-        <v>1031</v>
-      </c>
-      <c r="I5" s="14" t="s">
-        <v>948</v>
-      </c>
-      <c r="J5" s="14" t="s">
-        <v>1015</v>
+      <c r="H5" s="36" t="s">
+        <v>1030</v>
+      </c>
+      <c r="I5" s="13" t="s">
+        <v>947</v>
+      </c>
+      <c r="J5" s="13" t="s">
+        <v>1014</v>
       </c>
       <c r="K5" s="11" t="s">
         <v>819</v>
       </c>
-      <c r="L5" s="13">
+      <c r="L5" s="12">
         <v>7</v>
       </c>
-      <c r="M5" s="13" t="s">
+      <c r="M5" s="12" t="s">
         <v>801</v>
       </c>
-      <c r="N5" s="13" t="s">
+      <c r="N5" s="12" t="s">
         <v>820</v>
       </c>
-      <c r="O5" s="13" t="s">
+      <c r="O5" s="12" t="s">
         <v>822</v>
       </c>
-      <c r="P5" s="13" t="s">
+      <c r="P5" s="12" t="s">
         <v>149</v>
       </c>
-      <c r="Q5" s="13" t="s">
+      <c r="Q5" s="12" t="s">
         <v>823</v>
       </c>
-      <c r="R5" s="17" t="s">
+      <c r="R5" s="16" t="s">
         <v>765</v>
       </c>
-      <c r="S5" s="17" t="e">
+      <c r="S5" s="16" t="e">
         <f t="shared" ca="1" si="1"/>
         <v>#VALUE!</v>
       </c>
@@ -5230,10 +5213,10 @@
       <c r="V5" s="7" t="s">
         <v>825</v>
       </c>
-      <c r="W5" s="13" t="s">
+      <c r="W5" s="12" t="s">
         <v>577</v>
       </c>
-      <c r="X5" s="13" t="s">
+      <c r="X5" s="12" t="s">
         <v>796</v>
       </c>
       <c r="Y5" s="7" t="s">
@@ -5245,7 +5228,7 @@
       <c r="AA5" s="7" t="s">
         <v>490</v>
       </c>
-      <c r="AB5" s="13" t="s">
+      <c r="AB5" s="12" t="s">
         <v>826</v>
       </c>
       <c r="AE5" s="7" t="s">
@@ -5275,13 +5258,13 @@
       <c r="AN5" s="7" t="s">
         <v>236</v>
       </c>
-      <c r="AO5" s="13">
+      <c r="AO5" s="12">
         <v>35</v>
       </c>
-      <c r="AP5" s="13">
+      <c r="AP5" s="12">
         <v>157</v>
       </c>
-      <c r="AQ5" s="13" t="s">
+      <c r="AQ5" s="12" t="s">
         <v>164</v>
       </c>
       <c r="AR5" s="7" t="s">
@@ -5294,24 +5277,24 @@
         <v>167</v>
       </c>
       <c r="AU5" s="7" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="AV5" s="7" t="s">
         <v>823</v>
       </c>
-      <c r="AW5" s="15" t="s">
-        <v>949</v>
-      </c>
-      <c r="AX5" s="35" t="s">
-        <v>1039</v>
+      <c r="AW5" s="14" t="s">
+        <v>948</v>
+      </c>
+      <c r="AX5" s="34" t="s">
+        <v>1038</v>
       </c>
       <c r="AY5" s="7" t="s">
-        <v>915</v>
-      </c>
-      <c r="BA5" s="13">
+        <v>914</v>
+      </c>
+      <c r="BA5" s="12">
         <v>2</v>
       </c>
-      <c r="BB5" s="13">
+      <c r="BB5" s="12">
         <v>6</v>
       </c>
       <c r="BC5" s="7" t="s">
@@ -5323,17 +5306,17 @@
       <c r="BE5" s="11" t="s">
         <v>490</v>
       </c>
-      <c r="BF5" s="13">
+      <c r="BF5" s="12">
         <v>65141</v>
       </c>
       <c r="BG5" s="7" t="s">
         <v>161</v>
       </c>
-      <c r="BH5" s="13" t="s">
+      <c r="BH5" s="12" t="s">
         <v>162</v>
       </c>
-      <c r="BI5" s="13" t="s">
-        <v>916</v>
+      <c r="BI5" s="12" t="s">
+        <v>915</v>
       </c>
       <c r="BJ5" s="7" t="s">
         <v>174</v>
@@ -5342,39 +5325,39 @@
         <v>865</v>
       </c>
       <c r="BL5" s="7" t="s">
+        <v>916</v>
+      </c>
+      <c r="BM5" s="7" t="s">
         <v>917</v>
       </c>
-      <c r="BM5" s="7" t="s">
-        <v>918</v>
-      </c>
-      <c r="BN5" s="13" t="s">
+      <c r="BN5" s="12" t="s">
         <v>910</v>
       </c>
-      <c r="BO5" s="21">
+      <c r="BO5" s="20">
         <v>6700000</v>
       </c>
       <c r="BP5" s="7" t="s">
         <v>911</v>
       </c>
       <c r="BR5" s="11" t="s">
+        <v>918</v>
+      </c>
+      <c r="BS5" s="7" t="s">
         <v>919</v>
       </c>
-      <c r="BS5" s="7" t="s">
+      <c r="BT5" s="14" t="s">
+        <v>949</v>
+      </c>
+      <c r="BU5" s="7" t="s">
         <v>920</v>
       </c>
-      <c r="BT5" s="15" t="s">
-        <v>950</v>
-      </c>
-      <c r="BU5" s="7" t="s">
-        <v>921</v>
-      </c>
       <c r="BV5" s="7" t="s">
-        <v>915</v>
-      </c>
-      <c r="BW5" s="13">
+        <v>914</v>
+      </c>
+      <c r="BW5" s="12">
         <v>2</v>
       </c>
-      <c r="BX5" s="13">
+      <c r="BX5" s="12">
         <v>6</v>
       </c>
       <c r="BY5" s="7" t="s">
@@ -5386,7 +5369,7 @@
       <c r="CA5" s="11" t="s">
         <v>156</v>
       </c>
-      <c r="CB5" s="13">
+      <c r="CB5" s="12">
         <v>65141</v>
       </c>
       <c r="CC5" s="7" t="s">
@@ -5395,8 +5378,8 @@
       <c r="CD5" s="7" t="s">
         <v>162</v>
       </c>
-      <c r="CE5" s="13" t="s">
-        <v>922</v>
+      <c r="CE5" s="12" t="s">
+        <v>921</v>
       </c>
       <c r="CF5" s="7" t="s">
         <v>183</v>
@@ -5405,12 +5388,12 @@
         <v>500</v>
       </c>
       <c r="CH5" s="7" t="s">
-        <v>923</v>
+        <v>922</v>
       </c>
       <c r="CI5" s="7" t="s">
-        <v>915</v>
-      </c>
-      <c r="CJ5" s="19"/>
+        <v>914</v>
+      </c>
+      <c r="CJ5" s="18"/>
       <c r="CK5" s="7">
         <v>1500000</v>
       </c>
@@ -5418,7 +5401,7 @@
         <v>912</v>
       </c>
       <c r="CO5" s="11"/>
-      <c r="CP5" s="13"/>
+      <c r="CP5" s="12"/>
       <c r="CU5" s="11"/>
       <c r="CV5" s="11"/>
       <c r="CW5" s="11"/>
@@ -5427,18 +5410,12 @@
       <c r="DG5" s="7" t="s">
         <v>186</v>
       </c>
-      <c r="DH5" s="7" t="s">
-        <v>835</v>
-      </c>
-      <c r="DI5" s="7" t="s">
-        <v>913</v>
-      </c>
     </row>
     <row r="6" spans="1:113" s="7" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="13">
+      <c r="A6" s="12">
         <v>5</v>
       </c>
-      <c r="B6" s="15" t="s">
+      <c r="B6" s="14" t="s">
         <v>832</v>
       </c>
       <c r="C6" s="7" t="s">
@@ -5450,46 +5427,46 @@
       <c r="E6" s="7" t="s">
         <v>803</v>
       </c>
-      <c r="F6" s="14" t="s">
-        <v>928</v>
-      </c>
-      <c r="G6" s="14" t="s">
+      <c r="F6" s="13" t="s">
+        <v>927</v>
+      </c>
+      <c r="G6" s="13" t="s">
         <v>807</v>
       </c>
-      <c r="H6" s="37" t="s">
-        <v>1032</v>
-      </c>
-      <c r="I6" s="13" t="s">
-        <v>951</v>
-      </c>
-      <c r="J6" s="13" t="s">
+      <c r="H6" s="36" t="s">
+        <v>1031</v>
+      </c>
+      <c r="I6" s="12" t="s">
+        <v>950</v>
+      </c>
+      <c r="J6" s="12" t="s">
         <v>225</v>
       </c>
       <c r="K6" s="7" t="s">
         <v>222</v>
       </c>
-      <c r="L6" s="13">
+      <c r="L6" s="12">
         <v>7</v>
       </c>
-      <c r="M6" s="13" t="s">
+      <c r="M6" s="12" t="s">
         <v>801</v>
       </c>
-      <c r="N6" s="13" t="s">
+      <c r="N6" s="12" t="s">
         <v>223</v>
       </c>
-      <c r="O6" s="13" t="s">
+      <c r="O6" s="12" t="s">
         <v>224</v>
       </c>
-      <c r="P6" s="13" t="s">
+      <c r="P6" s="12" t="s">
         <v>149</v>
       </c>
-      <c r="Q6" s="13" t="s">
+      <c r="Q6" s="12" t="s">
         <v>226</v>
       </c>
-      <c r="R6" s="17" t="s">
+      <c r="R6" s="16" t="s">
         <v>818</v>
       </c>
-      <c r="S6" s="17" t="e">
+      <c r="S6" s="16" t="e">
         <f t="shared" ca="1" si="1"/>
         <v>#VALUE!</v>
       </c>
@@ -5499,10 +5476,10 @@
       <c r="V6" s="7" t="s">
         <v>227</v>
       </c>
-      <c r="W6" s="13" t="s">
+      <c r="W6" s="12" t="s">
         <v>228</v>
       </c>
-      <c r="X6" s="13" t="s">
+      <c r="X6" s="12" t="s">
         <v>229</v>
       </c>
       <c r="Y6" s="7" t="s">
@@ -5514,7 +5491,7 @@
       <c r="AA6" s="7" t="s">
         <v>787</v>
       </c>
-      <c r="AB6" s="13">
+      <c r="AB6" s="12">
         <v>65153</v>
       </c>
       <c r="AC6" s="7" t="s">
@@ -5553,13 +5530,13 @@
       <c r="AN6" s="7" t="s">
         <v>236</v>
       </c>
-      <c r="AO6" s="13" t="s">
+      <c r="AO6" s="12" t="s">
         <v>237</v>
       </c>
-      <c r="AP6" s="13">
+      <c r="AP6" s="12">
         <v>145</v>
       </c>
-      <c r="AQ6" s="13" t="s">
+      <c r="AQ6" s="12" t="s">
         <v>238</v>
       </c>
       <c r="AR6" s="7" t="s">
@@ -5577,8 +5554,8 @@
       <c r="AV6" s="7" t="s">
         <v>241</v>
       </c>
-      <c r="AW6" s="15" t="s">
-        <v>952</v>
+      <c r="AW6" s="14" t="s">
+        <v>951</v>
       </c>
       <c r="AX6" s="7" t="s">
         <v>242</v>
@@ -5586,10 +5563,10 @@
       <c r="AY6" s="7" t="s">
         <v>227</v>
       </c>
-      <c r="BA6" s="13" t="s">
+      <c r="BA6" s="12" t="s">
         <v>228</v>
       </c>
-      <c r="BB6" s="13" t="s">
+      <c r="BB6" s="12" t="s">
         <v>229</v>
       </c>
       <c r="BC6" s="7" t="s">
@@ -5601,16 +5578,16 @@
       <c r="BE6" s="11" t="s">
         <v>787</v>
       </c>
-      <c r="BF6" s="13">
+      <c r="BF6" s="12">
         <v>65153</v>
       </c>
       <c r="BG6" s="7" t="s">
         <v>161</v>
       </c>
-      <c r="BH6" s="13" t="s">
+      <c r="BH6" s="12" t="s">
         <v>162</v>
       </c>
-      <c r="BI6" s="13" t="s">
+      <c r="BI6" s="12" t="s">
         <v>243</v>
       </c>
       <c r="BJ6" s="7" t="s">
@@ -5626,10 +5603,10 @@
       <c r="BM6" s="7" t="s">
         <v>246</v>
       </c>
-      <c r="BN6" s="13" t="s">
+      <c r="BN6" s="12" t="s">
         <v>247</v>
       </c>
-      <c r="BO6" s="21" t="s">
+      <c r="BO6" s="20" t="s">
         <v>248</v>
       </c>
       <c r="BP6" s="7" t="s">
@@ -5644,8 +5621,8 @@
       <c r="BS6" s="7" t="s">
         <v>252</v>
       </c>
-      <c r="BT6" s="15" t="s">
-        <v>953</v>
+      <c r="BT6" s="14" t="s">
+        <v>952</v>
       </c>
       <c r="BU6" s="7" t="s">
         <v>253</v>
@@ -5653,10 +5630,10 @@
       <c r="BV6" s="7" t="s">
         <v>227</v>
       </c>
-      <c r="BW6" s="13" t="s">
+      <c r="BW6" s="12" t="s">
         <v>228</v>
       </c>
-      <c r="BX6" s="13" t="s">
+      <c r="BX6" s="12" t="s">
         <v>229</v>
       </c>
       <c r="BY6" s="7" t="s">
@@ -5668,7 +5645,7 @@
       <c r="CA6" s="11" t="s">
         <v>787</v>
       </c>
-      <c r="CB6" s="13">
+      <c r="CB6" s="12">
         <v>65153</v>
       </c>
       <c r="CC6" s="7" t="s">
@@ -5677,7 +5654,7 @@
       <c r="CD6" s="7" t="s">
         <v>162</v>
       </c>
-      <c r="CE6" s="13" t="s">
+      <c r="CE6" s="12" t="s">
         <v>232</v>
       </c>
       <c r="CF6" s="7" t="s">
@@ -5692,7 +5669,7 @@
       <c r="CI6" s="7" t="s">
         <v>255</v>
       </c>
-      <c r="CJ6" s="13" t="s">
+      <c r="CJ6" s="12" t="s">
         <v>256</v>
       </c>
       <c r="CK6" s="7" t="s">
@@ -5707,13 +5684,13 @@
       <c r="CN6" s="7" t="s">
         <v>841</v>
       </c>
-      <c r="CP6" s="13"/>
+      <c r="CP6" s="12"/>
     </row>
     <row r="7" spans="1:113" s="7" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="13">
+      <c r="A7" s="12">
         <v>6</v>
       </c>
-      <c r="B7" s="15" t="s">
+      <c r="B7" s="14" t="s">
         <v>832</v>
       </c>
       <c r="C7" s="7" t="s">
@@ -5725,44 +5702,44 @@
       <c r="E7" s="7" t="s">
         <v>803</v>
       </c>
-      <c r="F7" s="14" t="s">
-        <v>929</v>
-      </c>
-      <c r="G7" s="14" t="s">
+      <c r="F7" s="13" t="s">
+        <v>928</v>
+      </c>
+      <c r="G7" s="13" t="s">
         <v>802</v>
       </c>
-      <c r="H7" s="15"/>
-      <c r="I7" s="14" t="s">
-        <v>954</v>
-      </c>
-      <c r="J7" s="14" t="s">
-        <v>1009</v>
+      <c r="H7" s="14"/>
+      <c r="I7" s="13" t="s">
+        <v>953</v>
+      </c>
+      <c r="J7" s="13" t="s">
+        <v>1008</v>
       </c>
       <c r="K7" s="7" t="s">
         <v>282</v>
       </c>
-      <c r="L7" s="13">
+      <c r="L7" s="12">
         <v>7</v>
       </c>
-      <c r="M7" s="13" t="s">
+      <c r="M7" s="12" t="s">
         <v>801</v>
       </c>
-      <c r="N7" s="13" t="s">
+      <c r="N7" s="12" t="s">
         <v>283</v>
       </c>
-      <c r="O7" s="13" t="s">
+      <c r="O7" s="12" t="s">
         <v>284</v>
       </c>
-      <c r="P7" s="13" t="s">
+      <c r="P7" s="12" t="s">
         <v>286</v>
       </c>
-      <c r="Q7" s="13" t="s">
+      <c r="Q7" s="12" t="s">
         <v>226</v>
       </c>
-      <c r="R7" s="17" t="s">
+      <c r="R7" s="16" t="s">
         <v>760</v>
       </c>
-      <c r="S7" s="17" t="e">
+      <c r="S7" s="16" t="e">
         <f t="shared" ca="1" si="1"/>
         <v>#VALUE!</v>
       </c>
@@ -5775,10 +5752,10 @@
       <c r="V7" s="7" t="s">
         <v>804</v>
       </c>
-      <c r="W7" s="13">
+      <c r="W7" s="12">
         <v>3</v>
       </c>
-      <c r="X7" s="13">
+      <c r="X7" s="12">
         <v>12</v>
       </c>
       <c r="Y7" s="7" t="s">
@@ -5790,7 +5767,7 @@
       <c r="AA7" s="7" t="s">
         <v>490</v>
       </c>
-      <c r="AB7" s="13">
+      <c r="AB7" s="12">
         <v>65144</v>
       </c>
       <c r="AC7" s="7" t="s">
@@ -5823,13 +5800,13 @@
       <c r="AN7" s="7" t="s">
         <v>236</v>
       </c>
-      <c r="AO7" s="13">
+      <c r="AO7" s="12">
         <v>50</v>
       </c>
-      <c r="AP7" s="13">
+      <c r="AP7" s="12">
         <v>163</v>
       </c>
-      <c r="AQ7" s="13" t="s">
+      <c r="AQ7" s="12" t="s">
         <v>164</v>
       </c>
       <c r="AR7" s="7" t="s">
@@ -5847,8 +5824,8 @@
       <c r="AV7" s="7" t="s">
         <v>226</v>
       </c>
-      <c r="AW7" s="15" t="s">
-        <v>955</v>
+      <c r="AW7" s="14" t="s">
+        <v>954</v>
       </c>
       <c r="AX7" s="7" t="s">
         <v>297</v>
@@ -5856,10 +5833,10 @@
       <c r="AY7" s="7" t="s">
         <v>854</v>
       </c>
-      <c r="BA7" s="13">
+      <c r="BA7" s="12">
         <v>3</v>
       </c>
-      <c r="BB7" s="13">
+      <c r="BB7" s="12">
         <v>12</v>
       </c>
       <c r="BC7" s="7" t="s">
@@ -5871,16 +5848,16 @@
       <c r="BE7" s="7" t="s">
         <v>490</v>
       </c>
-      <c r="BF7" s="13">
+      <c r="BF7" s="12">
         <v>65144</v>
       </c>
       <c r="BG7" s="7" t="s">
         <v>161</v>
       </c>
-      <c r="BH7" s="13" t="s">
+      <c r="BH7" s="12" t="s">
         <v>162</v>
       </c>
-      <c r="BI7" s="13" t="s">
+      <c r="BI7" s="12" t="s">
         <v>299</v>
       </c>
       <c r="BJ7" s="7" t="s">
@@ -5896,10 +5873,10 @@
       <c r="BM7" s="7" t="s">
         <v>873</v>
       </c>
-      <c r="BN7" s="13" t="s">
+      <c r="BN7" s="12" t="s">
         <v>304</v>
       </c>
-      <c r="BO7" s="21" t="s">
+      <c r="BO7" s="20" t="s">
         <v>305</v>
       </c>
       <c r="BP7" s="7" t="s">
@@ -5914,8 +5891,8 @@
       <c r="BS7" s="7" t="s">
         <v>226</v>
       </c>
-      <c r="BT7" s="15" t="s">
-        <v>956</v>
+      <c r="BT7" s="14" t="s">
+        <v>955</v>
       </c>
       <c r="BU7" s="7" t="s">
         <v>308</v>
@@ -5923,10 +5900,10 @@
       <c r="BV7" s="7" t="s">
         <v>854</v>
       </c>
-      <c r="BW7" s="13">
+      <c r="BW7" s="12">
         <v>3</v>
       </c>
-      <c r="BX7" s="13">
+      <c r="BX7" s="12">
         <v>12</v>
       </c>
       <c r="BY7" s="7" t="s">
@@ -5938,7 +5915,7 @@
       <c r="CA7" s="11" t="s">
         <v>490</v>
       </c>
-      <c r="CB7" s="13">
+      <c r="CB7" s="12">
         <v>65144</v>
       </c>
       <c r="CC7" s="7" t="s">
@@ -5947,7 +5924,7 @@
       <c r="CD7" s="7" t="s">
         <v>162</v>
       </c>
-      <c r="CE7" s="13" t="s">
+      <c r="CE7" s="12" t="s">
         <v>291</v>
       </c>
       <c r="CF7" s="7" t="s">
@@ -5962,7 +5939,7 @@
       <c r="CI7" s="7" t="s">
         <v>873</v>
       </c>
-      <c r="CJ7" s="13" t="s">
+      <c r="CJ7" s="12" t="s">
         <v>304</v>
       </c>
       <c r="CK7" s="7" t="s">
@@ -5980,7 +5957,7 @@
       <c r="CO7" s="11" t="s">
         <v>226</v>
       </c>
-      <c r="CP7" s="13">
+      <c r="CP7" s="12">
         <v>24521</v>
       </c>
       <c r="CQ7" s="7" t="s">
@@ -6039,294 +6016,294 @@
       </c>
     </row>
     <row r="8" spans="1:113" s="7" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="13">
+      <c r="A8" s="12">
         <v>7</v>
       </c>
-      <c r="B8" s="24" t="s">
-        <v>998</v>
-      </c>
-      <c r="C8" s="25" t="s">
+      <c r="B8" s="23" t="s">
         <v>997</v>
       </c>
-      <c r="D8" s="26" t="s">
+      <c r="C8" s="24" t="s">
+        <v>996</v>
+      </c>
+      <c r="D8" s="25" t="s">
+        <v>987</v>
+      </c>
+      <c r="E8" s="25" t="s">
         <v>988</v>
       </c>
-      <c r="E8" s="26" t="s">
+      <c r="F8" s="26" t="s">
         <v>989</v>
       </c>
-      <c r="F8" s="27" t="s">
+      <c r="G8" s="26" t="s">
         <v>990</v>
       </c>
-      <c r="G8" s="27" t="s">
+      <c r="H8" s="37" t="s">
+        <v>1033</v>
+      </c>
+      <c r="I8" s="26" t="s">
         <v>991</v>
       </c>
-      <c r="H8" s="38" t="s">
-        <v>1034</v>
-      </c>
-      <c r="I8" s="27" t="s">
+      <c r="J8" s="26" t="s">
         <v>992</v>
       </c>
-      <c r="J8" s="27" t="s">
+      <c r="K8" s="24" t="s">
+        <v>986</v>
+      </c>
+      <c r="L8" s="27">
+        <v>7</v>
+      </c>
+      <c r="M8" s="28" t="s">
+        <v>801</v>
+      </c>
+      <c r="N8" s="28" t="s">
         <v>993</v>
       </c>
-      <c r="K8" s="25" t="s">
-        <v>987</v>
-      </c>
-      <c r="L8" s="28">
-        <v>7</v>
-      </c>
-      <c r="M8" s="29" t="s">
-        <v>801</v>
-      </c>
-      <c r="N8" s="29" t="s">
+      <c r="O8" s="26" t="s">
         <v>994</v>
       </c>
-      <c r="O8" s="27" t="s">
+      <c r="P8" s="28" t="s">
+        <v>286</v>
+      </c>
+      <c r="Q8" s="28" t="s">
+        <v>593</v>
+      </c>
+      <c r="R8" s="29" t="s">
         <v>995</v>
       </c>
-      <c r="P8" s="29" t="s">
-        <v>286</v>
-      </c>
-      <c r="Q8" s="29" t="s">
-        <v>593</v>
-      </c>
-      <c r="R8" s="30" t="s">
-        <v>996</v>
-      </c>
-      <c r="S8" s="31" t="e">
+      <c r="S8" s="30" t="e">
         <f t="shared" ca="1" si="1"/>
         <v>#VALUE!</v>
       </c>
-      <c r="T8" s="25" t="s">
+      <c r="T8" s="24" t="s">
         <v>151</v>
       </c>
-      <c r="U8" s="26"/>
-      <c r="V8" s="26" t="s">
+      <c r="U8" s="25"/>
+      <c r="V8" s="25" t="s">
+        <v>1022</v>
+      </c>
+      <c r="W8" s="26" t="s">
+        <v>346</v>
+      </c>
+      <c r="X8" s="26" t="s">
+        <v>1018</v>
+      </c>
+      <c r="Y8" s="24" t="s">
+        <v>1019</v>
+      </c>
+      <c r="Z8" s="24" t="s">
+        <v>786</v>
+      </c>
+      <c r="AA8" s="24" t="s">
+        <v>787</v>
+      </c>
+      <c r="AB8" s="27">
+        <v>65152</v>
+      </c>
+      <c r="AC8" s="35" t="s">
+        <v>1020</v>
+      </c>
+      <c r="AD8" s="25" t="s">
+        <v>1020</v>
+      </c>
+      <c r="AE8" s="24" t="s">
+        <v>998</v>
+      </c>
+      <c r="AF8" s="24" t="s">
+        <v>1001</v>
+      </c>
+      <c r="AG8" s="25">
+        <v>1</v>
+      </c>
+      <c r="AH8" s="25">
+        <v>3</v>
+      </c>
+      <c r="AI8" s="25"/>
+      <c r="AJ8" s="25"/>
+      <c r="AK8" s="24" t="s">
+        <v>1021</v>
+      </c>
+      <c r="AL8" s="25" t="s">
+        <v>161</v>
+      </c>
+      <c r="AM8" s="25" t="s">
+        <v>162</v>
+      </c>
+      <c r="AN8" s="24" t="s">
+        <v>236</v>
+      </c>
+      <c r="AO8" s="27">
+        <v>49</v>
+      </c>
+      <c r="AP8" s="27">
+        <v>156</v>
+      </c>
+      <c r="AQ8" s="28" t="s">
+        <v>494</v>
+      </c>
+      <c r="AR8" s="24" t="s">
+        <v>1015</v>
+      </c>
+      <c r="AS8" s="24" t="s">
+        <v>166</v>
+      </c>
+      <c r="AT8" s="24" t="s">
+        <v>401</v>
+      </c>
+      <c r="AU8" s="24" t="s">
+        <v>998</v>
+      </c>
+      <c r="AV8" s="25" t="s">
+        <v>593</v>
+      </c>
+      <c r="AW8" s="31" t="s">
+        <v>999</v>
+      </c>
+      <c r="AX8" s="33" t="s">
+        <v>1000</v>
+      </c>
+      <c r="AY8" s="25" t="s">
+        <v>1022</v>
+      </c>
+      <c r="AZ8" s="25"/>
+      <c r="BA8" s="26" t="s">
+        <v>346</v>
+      </c>
+      <c r="BB8" s="26" t="s">
+        <v>1018</v>
+      </c>
+      <c r="BC8" s="24" t="s">
+        <v>1019</v>
+      </c>
+      <c r="BD8" s="24" t="s">
+        <v>786</v>
+      </c>
+      <c r="BE8" s="24" t="s">
+        <v>787</v>
+      </c>
+      <c r="BF8" s="27">
+        <v>65152</v>
+      </c>
+      <c r="BG8" s="25" t="s">
+        <v>161</v>
+      </c>
+      <c r="BH8" s="27" t="s">
+        <v>162</v>
+      </c>
+      <c r="BI8" s="26" t="s">
         <v>1023</v>
       </c>
-      <c r="W8" s="27" t="s">
-        <v>346</v>
-      </c>
-      <c r="X8" s="27" t="s">
-        <v>1019</v>
-      </c>
-      <c r="Y8" s="25" t="s">
-        <v>1020</v>
-      </c>
-      <c r="Z8" s="25" t="s">
-        <v>786</v>
-      </c>
-      <c r="AA8" s="25" t="s">
-        <v>787</v>
-      </c>
-      <c r="AB8" s="28">
-        <v>65152</v>
-      </c>
-      <c r="AC8" s="36" t="s">
-        <v>1021</v>
-      </c>
-      <c r="AD8" s="26" t="s">
-        <v>1021</v>
-      </c>
-      <c r="AE8" s="25" t="s">
-        <v>999</v>
-      </c>
-      <c r="AF8" s="25" t="s">
-        <v>1002</v>
-      </c>
-      <c r="AG8" s="26">
-        <v>1</v>
-      </c>
-      <c r="AH8" s="26">
-        <v>3</v>
-      </c>
-      <c r="AI8" s="26"/>
-      <c r="AJ8" s="26"/>
-      <c r="AK8" s="25" t="s">
-        <v>1022</v>
-      </c>
-      <c r="AL8" s="26" t="s">
-        <v>161</v>
-      </c>
-      <c r="AM8" s="26" t="s">
-        <v>162</v>
-      </c>
-      <c r="AN8" s="25" t="s">
-        <v>236</v>
-      </c>
-      <c r="AO8" s="28">
-        <v>49</v>
-      </c>
-      <c r="AP8" s="28">
-        <v>156</v>
-      </c>
-      <c r="AQ8" s="29" t="s">
-        <v>494</v>
-      </c>
-      <c r="AR8" s="25" t="s">
-        <v>1016</v>
-      </c>
-      <c r="AS8" s="25" t="s">
-        <v>166</v>
-      </c>
-      <c r="AT8" s="25" t="s">
-        <v>401</v>
-      </c>
-      <c r="AU8" s="25" t="s">
-        <v>999</v>
-      </c>
-      <c r="AV8" s="26" t="s">
-        <v>593</v>
-      </c>
-      <c r="AW8" s="32" t="s">
-        <v>1000</v>
-      </c>
-      <c r="AX8" s="34" t="s">
-        <v>1001</v>
-      </c>
-      <c r="AY8" s="26" t="s">
-        <v>1023</v>
-      </c>
-      <c r="AZ8" s="26"/>
-      <c r="BA8" s="27" t="s">
-        <v>346</v>
-      </c>
-      <c r="BB8" s="27" t="s">
-        <v>1019</v>
-      </c>
-      <c r="BC8" s="25" t="s">
-        <v>1020</v>
-      </c>
-      <c r="BD8" s="25" t="s">
-        <v>786</v>
-      </c>
-      <c r="BE8" s="25" t="s">
-        <v>787</v>
-      </c>
-      <c r="BF8" s="28">
-        <v>65152</v>
-      </c>
-      <c r="BG8" s="26" t="s">
-        <v>161</v>
-      </c>
-      <c r="BH8" s="28" t="s">
-        <v>162</v>
-      </c>
-      <c r="BI8" s="27" t="s">
-        <v>1024</v>
-      </c>
-      <c r="BJ8" s="25" t="s">
+      <c r="BJ8" s="24" t="s">
         <v>183</v>
       </c>
-      <c r="BK8" s="25" t="s">
+      <c r="BK8" s="24" t="s">
         <v>500</v>
       </c>
-      <c r="BL8" s="26" t="str">
+      <c r="BL8" s="25" t="str">
         <f t="shared" si="0"/>
         <v>WIRASWASTA</v>
       </c>
-      <c r="BM8" s="26" t="s">
+      <c r="BM8" s="25" t="s">
+        <v>1024</v>
+      </c>
+      <c r="BN8" s="26" t="s">
         <v>1025</v>
       </c>
-      <c r="BN8" s="27" t="s">
+      <c r="BO8" s="32">
+        <v>30000000</v>
+      </c>
+      <c r="BP8" s="24" t="s">
         <v>1026</v>
       </c>
-      <c r="BO8" s="33">
-        <v>30000000</v>
-      </c>
-      <c r="BP8" s="25" t="s">
+      <c r="BQ8" s="25"/>
+      <c r="BR8" s="25" t="s">
+        <v>1001</v>
+      </c>
+      <c r="BS8" s="25" t="s">
+        <v>593</v>
+      </c>
+      <c r="BT8" s="31" t="s">
+        <v>1002</v>
+      </c>
+      <c r="BU8" s="33" t="s">
+        <v>1003</v>
+      </c>
+      <c r="BV8" s="25" t="s">
+        <v>1022</v>
+      </c>
+      <c r="BW8" s="27" t="s">
+        <v>346</v>
+      </c>
+      <c r="BX8" s="27" t="s">
+        <v>1018</v>
+      </c>
+      <c r="BY8" s="25" t="s">
+        <v>1019</v>
+      </c>
+      <c r="BZ8" s="25" t="s">
+        <v>786</v>
+      </c>
+      <c r="CA8" s="24" t="s">
+        <v>787</v>
+      </c>
+      <c r="CB8" s="27">
+        <v>65152</v>
+      </c>
+      <c r="CC8" s="25" t="s">
+        <v>161</v>
+      </c>
+      <c r="CD8" s="25" t="s">
+        <v>162</v>
+      </c>
+      <c r="CE8" s="26" t="s">
         <v>1027</v>
       </c>
-      <c r="BQ8" s="26"/>
-      <c r="BR8" s="26" t="s">
-        <v>1002</v>
-      </c>
-      <c r="BS8" s="26" t="s">
-        <v>593</v>
-      </c>
-      <c r="BT8" s="32" t="s">
-        <v>1003</v>
-      </c>
-      <c r="BU8" s="34" t="s">
-        <v>1004</v>
-      </c>
-      <c r="BV8" s="26" t="s">
-        <v>1023</v>
-      </c>
-      <c r="BW8" s="28" t="s">
-        <v>346</v>
-      </c>
-      <c r="BX8" s="28" t="s">
-        <v>1019</v>
-      </c>
-      <c r="BY8" s="26" t="s">
-        <v>1020</v>
-      </c>
-      <c r="BZ8" s="26" t="s">
-        <v>786</v>
-      </c>
-      <c r="CA8" s="25" t="s">
-        <v>787</v>
-      </c>
-      <c r="CB8" s="28">
-        <v>65152</v>
-      </c>
-      <c r="CC8" s="26" t="s">
-        <v>161</v>
-      </c>
-      <c r="CD8" s="26" t="s">
-        <v>162</v>
-      </c>
-      <c r="CE8" s="27" t="s">
-        <v>1028</v>
-      </c>
-      <c r="CF8" s="25" t="s">
+      <c r="CF8" s="24" t="s">
         <v>183</v>
       </c>
-      <c r="CG8" s="25" t="s">
+      <c r="CG8" s="24" t="s">
         <v>891</v>
       </c>
-      <c r="CH8" s="25" t="s">
-        <v>152</v>
-      </c>
-      <c r="CI8" s="25" t="s">
-        <v>152</v>
-      </c>
-      <c r="CJ8" s="28"/>
-      <c r="CK8" s="26"/>
-      <c r="CL8" s="26" t="s">
+      <c r="CH8" s="24" t="s">
+        <v>152</v>
+      </c>
+      <c r="CI8" s="24" t="s">
+        <v>152</v>
+      </c>
+      <c r="CJ8" s="27"/>
+      <c r="CK8" s="25"/>
+      <c r="CL8" s="25" t="s">
+        <v>1016</v>
+      </c>
+      <c r="CM8" s="25" t="s">
         <v>1017</v>
       </c>
-      <c r="CM8" s="26" t="s">
-        <v>1018</v>
-      </c>
-      <c r="CN8" s="26"/>
-      <c r="CO8" s="25"/>
-      <c r="CP8" s="28"/>
-      <c r="CQ8" s="26"/>
-      <c r="CR8" s="26"/>
-      <c r="CS8" s="26"/>
-      <c r="CT8" s="26"/>
-      <c r="CU8" s="25"/>
-      <c r="CV8" s="25"/>
-      <c r="CW8" s="25"/>
-      <c r="CX8" s="26"/>
-      <c r="CY8" s="26"/>
-      <c r="CZ8" s="26"/>
-      <c r="DA8" s="26"/>
-      <c r="DB8" s="25"/>
-      <c r="DC8" s="25"/>
-      <c r="DD8" s="26"/>
-      <c r="DE8" s="26"/>
-      <c r="DF8" s="26"/>
-      <c r="DG8" s="26"/>
-      <c r="DH8" s="26"/>
+      <c r="CN8" s="25"/>
+      <c r="CO8" s="24"/>
+      <c r="CP8" s="27"/>
+      <c r="CQ8" s="25"/>
+      <c r="CR8" s="25"/>
+      <c r="CS8" s="25"/>
+      <c r="CT8" s="25"/>
+      <c r="CU8" s="24"/>
+      <c r="CV8" s="24"/>
+      <c r="CW8" s="24"/>
+      <c r="CX8" s="25"/>
+      <c r="CY8" s="25"/>
+      <c r="CZ8" s="25"/>
+      <c r="DA8" s="25"/>
+      <c r="DB8" s="24"/>
+      <c r="DC8" s="24"/>
+      <c r="DD8" s="25"/>
+      <c r="DE8" s="25"/>
+      <c r="DF8" s="25"/>
+      <c r="DG8" s="25"/>
+      <c r="DH8" s="25"/>
     </row>
     <row r="9" spans="1:113" s="7" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="13">
+      <c r="A9" s="12">
         <v>8</v>
       </c>
-      <c r="B9" s="15" t="s">
+      <c r="B9" s="14" t="s">
         <v>832</v>
       </c>
       <c r="C9" s="7" t="s">
@@ -6338,44 +6315,44 @@
       <c r="E9" s="7" t="s">
         <v>803</v>
       </c>
-      <c r="F9" s="14" t="s">
-        <v>930</v>
-      </c>
-      <c r="G9" s="14" t="s">
+      <c r="F9" s="13" t="s">
+        <v>929</v>
+      </c>
+      <c r="G9" s="13" t="s">
         <v>808</v>
       </c>
-      <c r="H9" s="15"/>
-      <c r="I9" s="14" t="s">
-        <v>957</v>
-      </c>
-      <c r="J9" s="14" t="s">
-        <v>1010</v>
+      <c r="H9" s="14"/>
+      <c r="I9" s="13" t="s">
+        <v>956</v>
+      </c>
+      <c r="J9" s="13" t="s">
+        <v>1009</v>
       </c>
       <c r="K9" s="7" t="s">
         <v>746</v>
       </c>
-      <c r="L9" s="13">
+      <c r="L9" s="12">
         <v>7</v>
       </c>
-      <c r="M9" s="13" t="s">
+      <c r="M9" s="12" t="s">
         <v>801</v>
       </c>
-      <c r="N9" s="13" t="s">
+      <c r="N9" s="12" t="s">
         <v>752</v>
       </c>
-      <c r="O9" s="13" t="s">
+      <c r="O9" s="12" t="s">
         <v>390</v>
       </c>
-      <c r="P9" s="13" t="s">
+      <c r="P9" s="12" t="s">
         <v>149</v>
       </c>
-      <c r="Q9" s="13" t="s">
+      <c r="Q9" s="12" t="s">
         <v>226</v>
       </c>
-      <c r="R9" s="17" t="s">
+      <c r="R9" s="16" t="s">
         <v>762</v>
       </c>
-      <c r="S9" s="17" t="e">
+      <c r="S9" s="16" t="e">
         <f t="shared" ca="1" si="1"/>
         <v>#VALUE!</v>
       </c>
@@ -6385,10 +6362,10 @@
       <c r="V9" s="7" t="s">
         <v>772</v>
       </c>
-      <c r="W9" s="13" t="s">
+      <c r="W9" s="12" t="s">
         <v>393</v>
       </c>
-      <c r="X9" s="13" t="s">
+      <c r="X9" s="12" t="s">
         <v>394</v>
       </c>
       <c r="Y9" s="7" t="s">
@@ -6400,7 +6377,7 @@
       <c r="AA9" s="7" t="s">
         <v>490</v>
       </c>
-      <c r="AB9" s="13">
+      <c r="AB9" s="12">
         <v>65141</v>
       </c>
       <c r="AC9" s="7" t="s">
@@ -6410,10 +6387,10 @@
         <v>396</v>
       </c>
       <c r="AE9" s="7" t="s">
+        <v>957</v>
+      </c>
+      <c r="AF9" s="7" t="s">
         <v>958</v>
-      </c>
-      <c r="AF9" s="7" t="s">
-        <v>959</v>
       </c>
       <c r="AG9" s="7">
         <v>1</v>
@@ -6439,13 +6416,13 @@
       <c r="AN9" s="7" t="s">
         <v>829</v>
       </c>
-      <c r="AO9" s="13">
+      <c r="AO9" s="12">
         <v>60</v>
       </c>
-      <c r="AP9" s="13">
+      <c r="AP9" s="12">
         <v>145</v>
       </c>
-      <c r="AQ9" s="13" t="s">
+      <c r="AQ9" s="12" t="s">
         <v>238</v>
       </c>
       <c r="AR9" s="7" t="s">
@@ -6463,19 +6440,19 @@
       <c r="AV9" s="7" t="s">
         <v>850</v>
       </c>
-      <c r="AW9" s="15" t="s">
-        <v>960</v>
-      </c>
-      <c r="AX9" s="35" t="s">
-        <v>1007</v>
+      <c r="AW9" s="14" t="s">
+        <v>959</v>
+      </c>
+      <c r="AX9" s="34" t="s">
+        <v>1006</v>
       </c>
       <c r="AY9" s="7" t="s">
         <v>855</v>
       </c>
-      <c r="BA9" s="13" t="s">
+      <c r="BA9" s="12" t="s">
         <v>393</v>
       </c>
-      <c r="BB9" s="13" t="s">
+      <c r="BB9" s="12" t="s">
         <v>394</v>
       </c>
       <c r="BC9" s="7" t="s">
@@ -6487,16 +6464,16 @@
       <c r="BE9" s="11" t="s">
         <v>490</v>
       </c>
-      <c r="BF9" s="13">
+      <c r="BF9" s="12">
         <v>65141</v>
       </c>
       <c r="BG9" s="7" t="s">
         <v>161</v>
       </c>
-      <c r="BH9" s="13" t="s">
+      <c r="BH9" s="12" t="s">
         <v>162</v>
       </c>
-      <c r="BI9" s="13" t="s">
+      <c r="BI9" s="12" t="s">
         <v>405</v>
       </c>
       <c r="BJ9" s="7" t="s">
@@ -6512,8 +6489,8 @@
       <c r="BM9" s="7" t="s">
         <v>874</v>
       </c>
-      <c r="BN9" s="13"/>
-      <c r="BO9" s="21" t="s">
+      <c r="BN9" s="12"/>
+      <c r="BO9" s="20" t="s">
         <v>409</v>
       </c>
       <c r="BP9" s="7" t="s">
@@ -6528,19 +6505,19 @@
       <c r="BS9" s="7" t="s">
         <v>885</v>
       </c>
-      <c r="BT9" s="15" t="s">
-        <v>961</v>
-      </c>
-      <c r="BU9" s="35" t="s">
-        <v>1008</v>
+      <c r="BT9" s="14" t="s">
+        <v>960</v>
+      </c>
+      <c r="BU9" s="34" t="s">
+        <v>1007</v>
       </c>
       <c r="BV9" s="7" t="s">
         <v>855</v>
       </c>
-      <c r="BW9" s="13" t="s">
+      <c r="BW9" s="12" t="s">
         <v>393</v>
       </c>
-      <c r="BX9" s="13" t="s">
+      <c r="BX9" s="12" t="s">
         <v>394</v>
       </c>
       <c r="BY9" s="7" t="s">
@@ -6552,7 +6529,7 @@
       <c r="CA9" s="11" t="s">
         <v>490</v>
       </c>
-      <c r="CB9" s="13">
+      <c r="CB9" s="12">
         <v>65141</v>
       </c>
       <c r="CC9" s="7" t="s">
@@ -6561,7 +6538,7 @@
       <c r="CD9" s="7" t="s">
         <v>162</v>
       </c>
-      <c r="CE9" s="13" t="s">
+      <c r="CE9" s="12" t="s">
         <v>396</v>
       </c>
       <c r="CF9" s="7" t="s">
@@ -6576,7 +6553,7 @@
       <c r="CI9" s="7" t="s">
         <v>898</v>
       </c>
-      <c r="CJ9" s="13"/>
+      <c r="CJ9" s="12"/>
       <c r="CK9" s="7" t="s">
         <v>416</v>
       </c>
@@ -6589,13 +6566,13 @@
       <c r="CN9" s="7" t="s">
         <v>841</v>
       </c>
-      <c r="CP9" s="13"/>
+      <c r="CP9" s="12"/>
     </row>
     <row r="10" spans="1:113" s="7" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="13">
+      <c r="A10" s="12">
         <v>9</v>
       </c>
-      <c r="B10" s="15" t="s">
+      <c r="B10" s="14" t="s">
         <v>832</v>
       </c>
       <c r="C10" s="7" t="s">
@@ -6605,48 +6582,48 @@
         <v>836</v>
       </c>
       <c r="E10" s="7" t="s">
+        <v>961</v>
+      </c>
+      <c r="F10" s="13" t="s">
+        <v>930</v>
+      </c>
+      <c r="G10" s="13" t="s">
+        <v>811</v>
+      </c>
+      <c r="H10" s="36" t="s">
+        <v>1037</v>
+      </c>
+      <c r="I10" s="13" t="s">
         <v>962</v>
       </c>
-      <c r="F10" s="14" t="s">
-        <v>931</v>
-      </c>
-      <c r="G10" s="14" t="s">
-        <v>811</v>
-      </c>
-      <c r="H10" s="37" t="s">
-        <v>1038</v>
-      </c>
-      <c r="I10" s="14" t="s">
-        <v>963</v>
-      </c>
-      <c r="J10" s="14" t="s">
-        <v>1014</v>
+      <c r="J10" s="13" t="s">
+        <v>1013</v>
       </c>
       <c r="K10" s="7" t="s">
         <v>747</v>
       </c>
-      <c r="L10" s="13">
+      <c r="L10" s="12">
         <v>7</v>
       </c>
-      <c r="M10" s="13" t="s">
+      <c r="M10" s="12" t="s">
         <v>801</v>
       </c>
-      <c r="N10" s="13" t="s">
+      <c r="N10" s="12" t="s">
         <v>753</v>
       </c>
-      <c r="O10" s="13" t="s">
+      <c r="O10" s="12" t="s">
         <v>436</v>
       </c>
-      <c r="P10" s="13" t="s">
+      <c r="P10" s="12" t="s">
         <v>149</v>
       </c>
-      <c r="Q10" s="13" t="s">
+      <c r="Q10" s="12" t="s">
         <v>226</v>
       </c>
-      <c r="R10" s="17" t="s">
+      <c r="R10" s="16" t="s">
         <v>763</v>
       </c>
-      <c r="S10" s="17" t="e">
+      <c r="S10" s="16" t="e">
         <f t="shared" ca="1" si="1"/>
         <v>#VALUE!</v>
       </c>
@@ -6656,10 +6633,10 @@
       <c r="V10" s="7" t="s">
         <v>773</v>
       </c>
-      <c r="W10" s="13">
+      <c r="W10" s="12">
         <v>3</v>
       </c>
-      <c r="X10" s="13">
+      <c r="X10" s="12">
         <v>4</v>
       </c>
       <c r="Y10" s="7" t="s">
@@ -6671,7 +6648,7 @@
       <c r="AA10" s="7" t="s">
         <v>490</v>
       </c>
-      <c r="AB10" s="13">
+      <c r="AB10" s="12">
         <v>65143</v>
       </c>
       <c r="AC10" s="7" t="s">
@@ -6704,13 +6681,13 @@
       <c r="AN10" s="7" t="s">
         <v>236</v>
       </c>
-      <c r="AO10" s="13">
+      <c r="AO10" s="12">
         <v>60</v>
       </c>
-      <c r="AP10" s="13">
+      <c r="AP10" s="12">
         <v>160</v>
       </c>
-      <c r="AQ10" s="13" t="s">
+      <c r="AQ10" s="12" t="s">
         <v>164</v>
       </c>
       <c r="AR10" s="7" t="s">
@@ -6728,19 +6705,19 @@
       <c r="AV10" s="7" t="s">
         <v>851</v>
       </c>
-      <c r="AW10" s="15" t="s">
-        <v>964</v>
-      </c>
-      <c r="AX10" s="35" t="s">
+      <c r="AW10" s="14" t="s">
+        <v>963</v>
+      </c>
+      <c r="AX10" s="34" t="s">
         <v>449</v>
       </c>
       <c r="AY10" s="7" t="s">
         <v>856</v>
       </c>
-      <c r="BA10" s="13">
+      <c r="BA10" s="12">
         <v>3</v>
       </c>
-      <c r="BB10" s="13">
+      <c r="BB10" s="12">
         <v>4</v>
       </c>
       <c r="BC10" s="7" t="s">
@@ -6752,16 +6729,16 @@
       <c r="BE10" s="7" t="s">
         <v>862</v>
       </c>
-      <c r="BF10" s="13">
+      <c r="BF10" s="12">
         <v>65143</v>
       </c>
       <c r="BG10" s="7" t="s">
         <v>161</v>
       </c>
-      <c r="BH10" s="13" t="s">
+      <c r="BH10" s="12" t="s">
         <v>162</v>
       </c>
-      <c r="BI10" s="13" t="s">
+      <c r="BI10" s="12" t="s">
         <v>442</v>
       </c>
       <c r="BJ10" s="7" t="s">
@@ -6777,8 +6754,8 @@
       <c r="BM10" s="7" t="s">
         <v>875</v>
       </c>
-      <c r="BN10" s="13"/>
-      <c r="BO10" s="21">
+      <c r="BN10" s="12"/>
+      <c r="BO10" s="20">
         <v>600</v>
       </c>
       <c r="BP10" s="7" t="s">
@@ -6790,8 +6767,8 @@
       <c r="BS10" s="7" t="s">
         <v>886</v>
       </c>
-      <c r="BT10" s="15" t="s">
-        <v>965</v>
+      <c r="BT10" s="14" t="s">
+        <v>964</v>
       </c>
       <c r="BU10" s="7" t="s">
         <v>457</v>
@@ -6799,10 +6776,10 @@
       <c r="BV10" s="7" t="s">
         <v>856</v>
       </c>
-      <c r="BW10" s="13">
+      <c r="BW10" s="12">
         <v>3</v>
       </c>
-      <c r="BX10" s="13">
+      <c r="BX10" s="12">
         <v>4</v>
       </c>
       <c r="BY10" s="7" t="s">
@@ -6814,7 +6791,7 @@
       <c r="CA10" s="11" t="s">
         <v>490</v>
       </c>
-      <c r="CB10" s="13">
+      <c r="CB10" s="12">
         <v>65143</v>
       </c>
       <c r="CC10" s="7" t="s">
@@ -6823,7 +6800,7 @@
       <c r="CD10" s="7" t="s">
         <v>162</v>
       </c>
-      <c r="CE10" s="13" t="s">
+      <c r="CE10" s="12" t="s">
         <v>441</v>
       </c>
       <c r="CF10" s="7" t="s">
@@ -6838,7 +6815,7 @@
       <c r="CI10" s="7" t="s">
         <v>899</v>
       </c>
-      <c r="CJ10" s="13"/>
+      <c r="CJ10" s="12"/>
       <c r="CK10" s="7" t="s">
         <v>460</v>
       </c>
@@ -6848,13 +6825,13 @@
       <c r="CN10" s="7" t="s">
         <v>841</v>
       </c>
-      <c r="CP10" s="13"/>
+      <c r="CP10" s="12"/>
     </row>
     <row r="11" spans="1:113" s="7" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="13">
+      <c r="A11" s="12">
         <v>10</v>
       </c>
-      <c r="B11" s="15" t="s">
+      <c r="B11" s="14" t="s">
         <v>832</v>
       </c>
       <c r="C11" s="7" t="s">
@@ -6866,46 +6843,46 @@
       <c r="E11" s="7" t="s">
         <v>803</v>
       </c>
-      <c r="F11" s="14" t="s">
-        <v>932</v>
-      </c>
-      <c r="G11" s="14" t="s">
+      <c r="F11" s="13" t="s">
+        <v>931</v>
+      </c>
+      <c r="G11" s="13" t="s">
         <v>810</v>
       </c>
-      <c r="H11" s="37" t="s">
-        <v>1037</v>
-      </c>
-      <c r="I11" s="14" t="s">
-        <v>966</v>
-      </c>
-      <c r="J11" s="13" t="s">
+      <c r="H11" s="36" t="s">
+        <v>1036</v>
+      </c>
+      <c r="I11" s="13" t="s">
+        <v>965</v>
+      </c>
+      <c r="J11" s="12" t="s">
         <v>530</v>
       </c>
       <c r="K11" s="7" t="s">
         <v>748</v>
       </c>
-      <c r="L11" s="13">
+      <c r="L11" s="12">
         <v>7</v>
       </c>
-      <c r="M11" s="13" t="s">
+      <c r="M11" s="12" t="s">
         <v>801</v>
       </c>
-      <c r="N11" s="13" t="s">
+      <c r="N11" s="12" t="s">
         <v>754</v>
       </c>
-      <c r="O11" s="13" t="s">
+      <c r="O11" s="12" t="s">
         <v>529</v>
       </c>
-      <c r="P11" s="13" t="s">
+      <c r="P11" s="12" t="s">
         <v>149</v>
       </c>
-      <c r="Q11" s="13" t="s">
+      <c r="Q11" s="12" t="s">
         <v>757</v>
       </c>
-      <c r="R11" s="17" t="s">
+      <c r="R11" s="16" t="s">
         <v>764</v>
       </c>
-      <c r="S11" s="17" t="e">
+      <c r="S11" s="16" t="e">
         <f t="shared" ca="1" si="1"/>
         <v>#VALUE!</v>
       </c>
@@ -6915,10 +6892,10 @@
       <c r="V11" s="7" t="s">
         <v>774</v>
       </c>
-      <c r="W11" s="13" t="s">
+      <c r="W11" s="12" t="s">
         <v>533</v>
       </c>
-      <c r="X11" s="13" t="s">
+      <c r="X11" s="12" t="s">
         <v>534</v>
       </c>
       <c r="Y11" s="7" t="s">
@@ -6930,7 +6907,7 @@
       <c r="AA11" s="7" t="s">
         <v>490</v>
       </c>
-      <c r="AB11" s="13">
+      <c r="AB11" s="12">
         <v>65141</v>
       </c>
       <c r="AC11" s="7" t="s">
@@ -6940,10 +6917,10 @@
         <v>536</v>
       </c>
       <c r="AE11" s="7" t="s">
+        <v>966</v>
+      </c>
+      <c r="AF11" s="7" t="s">
         <v>967</v>
-      </c>
-      <c r="AF11" s="7" t="s">
-        <v>968</v>
       </c>
       <c r="AG11" s="7">
         <v>1</v>
@@ -6963,13 +6940,13 @@
       <c r="AN11" s="7" t="s">
         <v>236</v>
       </c>
-      <c r="AO11" s="13" t="s">
+      <c r="AO11" s="12" t="s">
         <v>540</v>
       </c>
-      <c r="AP11" s="13">
+      <c r="AP11" s="12">
         <v>158</v>
       </c>
-      <c r="AQ11" s="13" t="s">
+      <c r="AQ11" s="12" t="s">
         <v>541</v>
       </c>
       <c r="AR11" s="7" t="s">
@@ -6982,13 +6959,13 @@
         <v>167</v>
       </c>
       <c r="AU11" s="7" t="s">
-        <v>969</v>
+        <v>968</v>
       </c>
       <c r="AV11" s="7" t="s">
         <v>852</v>
       </c>
-      <c r="AW11" s="15" t="s">
-        <v>970</v>
+      <c r="AW11" s="14" t="s">
+        <v>969</v>
       </c>
       <c r="AX11" s="7" t="s">
         <v>543</v>
@@ -6996,10 +6973,10 @@
       <c r="AY11" s="7" t="s">
         <v>857</v>
       </c>
-      <c r="BA11" s="13" t="s">
+      <c r="BA11" s="12" t="s">
         <v>533</v>
       </c>
-      <c r="BB11" s="13" t="s">
+      <c r="BB11" s="12" t="s">
         <v>534</v>
       </c>
       <c r="BC11" s="7" t="s">
@@ -7011,16 +6988,16 @@
       <c r="BE11" s="11" t="s">
         <v>490</v>
       </c>
-      <c r="BF11" s="13">
+      <c r="BF11" s="12">
         <v>65141</v>
       </c>
       <c r="BG11" s="7" t="s">
         <v>161</v>
       </c>
-      <c r="BH11" s="13" t="s">
+      <c r="BH11" s="12" t="s">
         <v>162</v>
       </c>
-      <c r="BI11" s="13" t="s">
+      <c r="BI11" s="12" t="s">
         <v>545</v>
       </c>
       <c r="BJ11" s="7" t="s">
@@ -7036,10 +7013,10 @@
       <c r="BM11" s="7" t="s">
         <v>876</v>
       </c>
-      <c r="BN11" s="13" t="s">
+      <c r="BN11" s="12" t="s">
         <v>549</v>
       </c>
-      <c r="BO11" s="21" t="s">
+      <c r="BO11" s="20" t="s">
         <v>550</v>
       </c>
       <c r="BP11" s="7" t="s">
@@ -7051,8 +7028,8 @@
       <c r="BS11" s="7" t="s">
         <v>887</v>
       </c>
-      <c r="BT11" s="15" t="s">
-        <v>971</v>
+      <c r="BT11" s="14" t="s">
+        <v>970</v>
       </c>
       <c r="BU11" s="7" t="s">
         <v>554</v>
@@ -7060,10 +7037,10 @@
       <c r="BV11" s="7" t="s">
         <v>774</v>
       </c>
-      <c r="BW11" s="13" t="s">
+      <c r="BW11" s="12" t="s">
         <v>533</v>
       </c>
-      <c r="BX11" s="13" t="s">
+      <c r="BX11" s="12" t="s">
         <v>534</v>
       </c>
       <c r="BY11" s="7" t="s">
@@ -7075,7 +7052,7 @@
       <c r="CA11" s="11" t="s">
         <v>490</v>
       </c>
-      <c r="CB11" s="13">
+      <c r="CB11" s="12">
         <v>65141</v>
       </c>
       <c r="CC11" s="7" t="s">
@@ -7084,7 +7061,7 @@
       <c r="CD11" s="7" t="s">
         <v>162</v>
       </c>
-      <c r="CE11" s="13" t="s">
+      <c r="CE11" s="12" t="s">
         <v>536</v>
       </c>
       <c r="CF11" s="7" t="s">
@@ -7099,7 +7076,7 @@
       <c r="CI11" s="7" t="s">
         <v>900</v>
       </c>
-      <c r="CJ11" s="13" t="s">
+      <c r="CJ11" s="12" t="s">
         <v>152</v>
       </c>
       <c r="CK11" s="7" t="s">
@@ -7111,13 +7088,13 @@
       <c r="CN11" s="7" t="s">
         <v>841</v>
       </c>
-      <c r="CP11" s="13"/>
+      <c r="CP11" s="12"/>
     </row>
     <row r="12" spans="1:113" s="7" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="13">
+      <c r="A12" s="12">
         <v>11</v>
       </c>
-      <c r="B12" s="15" t="s">
+      <c r="B12" s="14" t="s">
         <v>832</v>
       </c>
       <c r="C12" s="7" t="s">
@@ -7129,44 +7106,44 @@
       <c r="E12" s="7" t="s">
         <v>803</v>
       </c>
-      <c r="F12" s="14" t="s">
-        <v>933</v>
-      </c>
-      <c r="G12" s="14" t="s">
+      <c r="F12" s="13" t="s">
+        <v>932</v>
+      </c>
+      <c r="G12" s="13" t="s">
         <v>805</v>
       </c>
-      <c r="H12" s="15"/>
-      <c r="I12" s="14" t="s">
-        <v>972</v>
-      </c>
-      <c r="J12" s="14" t="s">
-        <v>1011</v>
+      <c r="H12" s="14"/>
+      <c r="I12" s="13" t="s">
+        <v>971</v>
+      </c>
+      <c r="J12" s="13" t="s">
+        <v>1010</v>
       </c>
       <c r="K12" s="7" t="s">
         <v>745</v>
       </c>
-      <c r="L12" s="13">
+      <c r="L12" s="12">
         <v>7</v>
       </c>
-      <c r="M12" s="13" t="s">
+      <c r="M12" s="12" t="s">
         <v>801</v>
       </c>
-      <c r="N12" s="13" t="s">
+      <c r="N12" s="12" t="s">
         <v>751</v>
       </c>
-      <c r="O12" s="13" t="s">
+      <c r="O12" s="12" t="s">
         <v>342</v>
       </c>
-      <c r="P12" s="13" t="s">
+      <c r="P12" s="12" t="s">
         <v>149</v>
       </c>
-      <c r="Q12" s="13" t="s">
+      <c r="Q12" s="12" t="s">
         <v>226</v>
       </c>
-      <c r="R12" s="17" t="s">
+      <c r="R12" s="16" t="s">
         <v>761</v>
       </c>
-      <c r="S12" s="17" t="e">
+      <c r="S12" s="16" t="e">
         <f t="shared" ca="1" si="1"/>
         <v>#VALUE!</v>
       </c>
@@ -7179,10 +7156,10 @@
       <c r="V12" s="7" t="s">
         <v>771</v>
       </c>
-      <c r="W12" s="13" t="s">
+      <c r="W12" s="12" t="s">
         <v>346</v>
       </c>
-      <c r="X12" s="13" t="s">
+      <c r="X12" s="12" t="s">
         <v>347</v>
       </c>
       <c r="Y12" s="7" t="s">
@@ -7194,7 +7171,7 @@
       <c r="AA12" s="7" t="s">
         <v>490</v>
       </c>
-      <c r="AB12" s="13">
+      <c r="AB12" s="12">
         <v>65144</v>
       </c>
       <c r="AC12" s="7">
@@ -7204,7 +7181,7 @@
         <v>349</v>
       </c>
       <c r="AE12" s="7" t="s">
-        <v>973</v>
+        <v>972</v>
       </c>
       <c r="AF12" s="7" t="s">
         <v>792</v>
@@ -7227,13 +7204,13 @@
       <c r="AN12" s="7" t="s">
         <v>236</v>
       </c>
-      <c r="AO12" s="13" t="s">
+      <c r="AO12" s="12" t="s">
         <v>354</v>
       </c>
-      <c r="AP12" s="13" t="s">
+      <c r="AP12" s="12" t="s">
         <v>355</v>
       </c>
-      <c r="AQ12" s="13" t="s">
+      <c r="AQ12" s="12" t="s">
         <v>164</v>
       </c>
       <c r="AR12" s="7" t="s">
@@ -7251,19 +7228,19 @@
       <c r="AV12" s="7" t="s">
         <v>226</v>
       </c>
-      <c r="AW12" s="15" t="s">
-        <v>974</v>
-      </c>
-      <c r="AX12" s="35" t="s">
-        <v>1012</v>
+      <c r="AW12" s="14" t="s">
+        <v>973</v>
+      </c>
+      <c r="AX12" s="34" t="s">
+        <v>1011</v>
       </c>
       <c r="AY12" s="7" t="s">
         <v>771</v>
       </c>
-      <c r="BA12" s="13" t="s">
+      <c r="BA12" s="12" t="s">
         <v>346</v>
       </c>
-      <c r="BB12" s="13" t="s">
+      <c r="BB12" s="12" t="s">
         <v>347</v>
       </c>
       <c r="BC12" s="7" t="s">
@@ -7275,16 +7252,16 @@
       <c r="BE12" s="11" t="s">
         <v>490</v>
       </c>
-      <c r="BF12" s="13">
+      <c r="BF12" s="12">
         <v>65144</v>
       </c>
       <c r="BG12" s="7" t="s">
         <v>161</v>
       </c>
-      <c r="BH12" s="13" t="s">
+      <c r="BH12" s="12" t="s">
         <v>162</v>
       </c>
-      <c r="BI12" s="13" t="s">
+      <c r="BI12" s="12" t="s">
         <v>358</v>
       </c>
       <c r="BJ12" s="7" t="s">
@@ -7300,8 +7277,8 @@
       <c r="BM12" s="7" t="s">
         <v>877</v>
       </c>
-      <c r="BN12" s="13"/>
-      <c r="BO12" s="21" t="s">
+      <c r="BN12" s="12"/>
+      <c r="BO12" s="20" t="s">
         <v>362</v>
       </c>
       <c r="BP12" s="7" t="s">
@@ -7313,19 +7290,19 @@
       <c r="BS12" s="7" t="s">
         <v>226</v>
       </c>
-      <c r="BT12" s="15" t="s">
-        <v>975</v>
-      </c>
-      <c r="BU12" s="35" t="s">
-        <v>1013</v>
+      <c r="BT12" s="14" t="s">
+        <v>974</v>
+      </c>
+      <c r="BU12" s="34" t="s">
+        <v>1012</v>
       </c>
       <c r="BV12" s="7" t="s">
         <v>771</v>
       </c>
-      <c r="BW12" s="13" t="s">
+      <c r="BW12" s="12" t="s">
         <v>346</v>
       </c>
-      <c r="BX12" s="13" t="s">
+      <c r="BX12" s="12" t="s">
         <v>347</v>
       </c>
       <c r="BY12" s="7" t="s">
@@ -7337,7 +7314,7 @@
       <c r="CA12" s="11" t="s">
         <v>490</v>
       </c>
-      <c r="CB12" s="13">
+      <c r="CB12" s="12">
         <v>65144</v>
       </c>
       <c r="CC12" s="7" t="s">
@@ -7346,7 +7323,7 @@
       <c r="CD12" s="7" t="s">
         <v>162</v>
       </c>
-      <c r="CE12" s="13" t="s">
+      <c r="CE12" s="12" t="s">
         <v>349</v>
       </c>
       <c r="CF12" s="7" t="s">
@@ -7361,7 +7338,7 @@
       <c r="CI12" s="7" t="s">
         <v>152</v>
       </c>
-      <c r="CJ12" s="13"/>
+      <c r="CJ12" s="12"/>
       <c r="CK12" s="7" t="s">
         <v>152</v>
       </c>
@@ -7371,13 +7348,13 @@
       <c r="CN12" s="7" t="s">
         <v>841</v>
       </c>
-      <c r="CP12" s="13"/>
+      <c r="CP12" s="12"/>
     </row>
     <row r="13" spans="1:113" s="7" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="13">
+      <c r="A13" s="12">
         <v>12</v>
       </c>
-      <c r="B13" s="15" t="s">
+      <c r="B13" s="14" t="s">
         <v>833</v>
       </c>
       <c r="C13" s="7" t="s">
@@ -7387,50 +7364,50 @@
         <v>838</v>
       </c>
       <c r="E13" s="7" t="s">
+        <v>975</v>
+      </c>
+      <c r="F13" s="13" t="s">
+        <v>933</v>
+      </c>
+      <c r="G13" s="13" t="s">
+        <v>813</v>
+      </c>
+      <c r="H13" s="36" t="s">
+        <v>1034</v>
+      </c>
+      <c r="I13" s="13" t="s">
         <v>976</v>
       </c>
-      <c r="F13" s="14" t="s">
-        <v>934</v>
-      </c>
-      <c r="G13" s="14" t="s">
-        <v>813</v>
-      </c>
-      <c r="H13" s="37" t="s">
-        <v>1035</v>
-      </c>
-      <c r="I13" s="14" t="s">
-        <v>977</v>
-      </c>
-      <c r="J13" s="13" t="s">
+      <c r="J13" s="12" t="s">
         <v>485</v>
       </c>
       <c r="K13" s="7" t="s">
         <v>482</v>
       </c>
-      <c r="L13" s="13">
+      <c r="L13" s="12">
         <v>7</v>
       </c>
-      <c r="M13" s="13" t="s">
+      <c r="M13" s="12" t="s">
         <v>801</v>
       </c>
-      <c r="N13" s="13" t="s">
+      <c r="N13" s="12" t="s">
         <v>483</v>
       </c>
-      <c r="O13" s="13" t="s">
+      <c r="O13" s="12" t="s">
         <v>484</v>
       </c>
-      <c r="P13" s="13" t="s">
+      <c r="P13" s="12" t="s">
         <v>149</v>
       </c>
-      <c r="Q13" s="13" t="s">
+      <c r="Q13" s="12" t="s">
         <v>226</v>
       </c>
-      <c r="R13" s="17" t="s">
+      <c r="R13" s="16" t="s">
         <v>817</v>
       </c>
-      <c r="S13" s="17" t="str">
+      <c r="S13" s="16" t="str">
         <f t="shared" ref="S13:S15" ca="1" si="2">DATEDIF(R13, TODAY(), "Y") &amp; " Tahun " &amp; DATEDIF(R13, TODAY(), "YM") &amp; " Bulan " &amp; DATEDIF(R13, TODAY(), "MD") &amp; " Hari"</f>
-        <v>12 Tahun 5 Bulan 21 Hari</v>
+        <v>12 Tahun 6 Bulan 14 Hari</v>
       </c>
       <c r="T13" s="7" t="s">
         <v>151</v>
@@ -7438,10 +7415,10 @@
       <c r="V13" s="7" t="s">
         <v>486</v>
       </c>
-      <c r="W13" s="13" t="s">
+      <c r="W13" s="12" t="s">
         <v>346</v>
       </c>
-      <c r="X13" s="13" t="s">
+      <c r="X13" s="12" t="s">
         <v>487</v>
       </c>
       <c r="Y13" s="7" t="s">
@@ -7453,7 +7430,7 @@
       <c r="AA13" s="7" t="s">
         <v>490</v>
       </c>
-      <c r="AB13" s="13">
+      <c r="AB13" s="12">
         <v>65144</v>
       </c>
       <c r="AC13" s="7">
@@ -7492,13 +7469,13 @@
       <c r="AN13" s="7" t="s">
         <v>236</v>
       </c>
-      <c r="AO13" s="13">
+      <c r="AO13" s="12">
         <v>24</v>
       </c>
-      <c r="AP13" s="13">
+      <c r="AP13" s="12">
         <v>141</v>
       </c>
-      <c r="AQ13" s="13" t="s">
+      <c r="AQ13" s="12" t="s">
         <v>494</v>
       </c>
       <c r="AR13" s="7" t="s">
@@ -7516,8 +7493,8 @@
       <c r="AV13" s="7" t="s">
         <v>496</v>
       </c>
-      <c r="AW13" s="15" t="s">
-        <v>978</v>
+      <c r="AW13" s="14" t="s">
+        <v>977</v>
       </c>
       <c r="AX13" s="7" t="s">
         <v>497</v>
@@ -7525,10 +7502,10 @@
       <c r="AY13" s="7" t="s">
         <v>498</v>
       </c>
-      <c r="BA13" s="13" t="s">
+      <c r="BA13" s="12" t="s">
         <v>346</v>
       </c>
-      <c r="BB13" s="13" t="s">
+      <c r="BB13" s="12" t="s">
         <v>487</v>
       </c>
       <c r="BC13" s="7" t="s">
@@ -7540,16 +7517,16 @@
       <c r="BE13" s="11" t="s">
         <v>490</v>
       </c>
-      <c r="BF13" s="13">
+      <c r="BF13" s="12">
         <v>65144</v>
       </c>
       <c r="BG13" s="7" t="s">
         <v>161</v>
       </c>
-      <c r="BH13" s="13" t="s">
+      <c r="BH13" s="12" t="s">
         <v>162</v>
       </c>
-      <c r="BI13" s="13" t="s">
+      <c r="BI13" s="12" t="s">
         <v>499</v>
       </c>
       <c r="BJ13" s="7" t="s">
@@ -7565,10 +7542,10 @@
       <c r="BM13" s="7" t="s">
         <v>878</v>
       </c>
-      <c r="BN13" s="13">
+      <c r="BN13" s="12">
         <v>0</v>
       </c>
-      <c r="BO13" s="21" t="s">
+      <c r="BO13" s="20" t="s">
         <v>257</v>
       </c>
       <c r="BP13" s="7" t="s">
@@ -7580,8 +7557,8 @@
       <c r="BS13" s="7" t="s">
         <v>502</v>
       </c>
-      <c r="BT13" s="15" t="s">
-        <v>979</v>
+      <c r="BT13" s="14" t="s">
+        <v>978</v>
       </c>
       <c r="BU13" s="7" t="s">
         <v>503</v>
@@ -7589,10 +7566,10 @@
       <c r="BV13" s="7" t="s">
         <v>486</v>
       </c>
-      <c r="BW13" s="13" t="s">
+      <c r="BW13" s="12" t="s">
         <v>346</v>
       </c>
-      <c r="BX13" s="13" t="s">
+      <c r="BX13" s="12" t="s">
         <v>487</v>
       </c>
       <c r="BY13" s="7" t="s">
@@ -7604,7 +7581,7 @@
       <c r="CA13" s="11" t="s">
         <v>490</v>
       </c>
-      <c r="CB13" s="13">
+      <c r="CB13" s="12">
         <v>65144</v>
       </c>
       <c r="CC13" s="7" t="s">
@@ -7613,7 +7590,7 @@
       <c r="CD13" s="7" t="s">
         <v>162</v>
       </c>
-      <c r="CE13" s="13" t="s">
+      <c r="CE13" s="12" t="s">
         <v>504</v>
       </c>
       <c r="CF13" s="7" t="s">
@@ -7628,7 +7605,7 @@
       <c r="CI13" s="7" t="s">
         <v>506</v>
       </c>
-      <c r="CJ13" s="13">
+      <c r="CJ13" s="12">
         <v>0</v>
       </c>
       <c r="CK13" s="7" t="s">
@@ -7640,13 +7617,13 @@
       <c r="CN13" s="7" t="s">
         <v>841</v>
       </c>
-      <c r="CP13" s="13"/>
+      <c r="CP13" s="12"/>
     </row>
     <row r="14" spans="1:113" s="7" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="13">
+      <c r="A14" s="12">
         <v>13</v>
       </c>
-      <c r="B14" s="15" t="s">
+      <c r="B14" s="14" t="s">
         <v>832</v>
       </c>
       <c r="C14" s="7" t="s">
@@ -7658,46 +7635,46 @@
       <c r="E14" s="7" t="s">
         <v>803</v>
       </c>
-      <c r="F14" s="14" t="s">
-        <v>935</v>
-      </c>
-      <c r="G14" s="14" t="s">
+      <c r="F14" s="13" t="s">
+        <v>934</v>
+      </c>
+      <c r="G14" s="13" t="s">
         <v>806</v>
       </c>
-      <c r="H14" s="37" t="s">
-        <v>1030</v>
-      </c>
-      <c r="I14" s="14" t="s">
-        <v>980</v>
-      </c>
-      <c r="J14" s="14" t="s">
+      <c r="H14" s="36" t="s">
+        <v>1029</v>
+      </c>
+      <c r="I14" s="13" t="s">
+        <v>979</v>
+      </c>
+      <c r="J14" s="13" t="s">
         <v>148</v>
       </c>
       <c r="K14" s="7" t="s">
         <v>145</v>
       </c>
-      <c r="L14" s="13">
+      <c r="L14" s="12">
         <v>7</v>
       </c>
-      <c r="M14" s="13" t="s">
+      <c r="M14" s="12" t="s">
         <v>801</v>
       </c>
-      <c r="N14" s="13" t="s">
+      <c r="N14" s="12" t="s">
         <v>146</v>
       </c>
-      <c r="O14" s="13" t="s">
+      <c r="O14" s="12" t="s">
         <v>147</v>
       </c>
-      <c r="P14" s="13" t="s">
+      <c r="P14" s="12" t="s">
         <v>149</v>
       </c>
-      <c r="Q14" s="13" t="s">
+      <c r="Q14" s="12" t="s">
         <v>226</v>
       </c>
-      <c r="R14" s="17" t="s">
+      <c r="R14" s="16" t="s">
         <v>759</v>
       </c>
-      <c r="S14" s="17" t="e">
+      <c r="S14" s="16" t="e">
         <f t="shared" ca="1" si="2"/>
         <v>#VALUE!</v>
       </c>
@@ -7707,10 +7684,10 @@
       <c r="V14" s="7" t="s">
         <v>770</v>
       </c>
-      <c r="W14" s="13">
+      <c r="W14" s="12">
         <v>19</v>
       </c>
-      <c r="X14" s="13">
+      <c r="X14" s="12">
         <v>1</v>
       </c>
       <c r="Y14" s="7" t="s">
@@ -7722,7 +7699,7 @@
       <c r="AA14" s="7" t="s">
         <v>490</v>
       </c>
-      <c r="AB14" s="13">
+      <c r="AB14" s="12">
         <v>65143</v>
       </c>
       <c r="AC14" s="7" t="s">
@@ -7761,13 +7738,13 @@
       <c r="AN14" s="7" t="s">
         <v>236</v>
       </c>
-      <c r="AO14" s="13">
+      <c r="AO14" s="12">
         <v>63</v>
       </c>
-      <c r="AP14" s="13">
+      <c r="AP14" s="12">
         <v>155</v>
       </c>
-      <c r="AQ14" s="13" t="s">
+      <c r="AQ14" s="12" t="s">
         <v>164</v>
       </c>
       <c r="AR14" s="7" t="s">
@@ -7785,19 +7762,19 @@
       <c r="AV14" s="7" t="s">
         <v>853</v>
       </c>
-      <c r="AW14" s="15" t="s">
-        <v>981</v>
-      </c>
-      <c r="AX14" s="35" t="s">
+      <c r="AW14" s="14" t="s">
+        <v>980</v>
+      </c>
+      <c r="AX14" s="34" t="s">
         <v>170</v>
       </c>
       <c r="AY14" s="7" t="s">
         <v>770</v>
       </c>
-      <c r="BA14" s="13">
+      <c r="BA14" s="12">
         <v>19</v>
       </c>
-      <c r="BB14" s="13">
+      <c r="BB14" s="12">
         <v>1</v>
       </c>
       <c r="BC14" s="7" t="s">
@@ -7809,16 +7786,16 @@
       <c r="BE14" s="7" t="s">
         <v>490</v>
       </c>
-      <c r="BF14" s="13">
+      <c r="BF14" s="12">
         <v>65143</v>
       </c>
       <c r="BG14" s="7" t="s">
         <v>161</v>
       </c>
-      <c r="BH14" s="13" t="s">
+      <c r="BH14" s="12" t="s">
         <v>162</v>
       </c>
-      <c r="BI14" s="13" t="s">
+      <c r="BI14" s="12" t="s">
         <v>157</v>
       </c>
       <c r="BJ14" s="7" t="s">
@@ -7834,10 +7811,10 @@
       <c r="BM14" s="7" t="s">
         <v>152</v>
       </c>
-      <c r="BN14" s="13" t="s">
-        <v>152</v>
-      </c>
-      <c r="BO14" s="21">
+      <c r="BN14" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="BO14" s="20">
         <v>6000000</v>
       </c>
       <c r="BP14" s="7" t="s">
@@ -7847,24 +7824,24 @@
         <v>177</v>
       </c>
       <c r="BR14" s="7" t="s">
-        <v>982</v>
+        <v>981</v>
       </c>
       <c r="BS14" s="7" t="s">
         <v>226</v>
       </c>
-      <c r="BT14" s="15" t="s">
-        <v>983</v>
-      </c>
-      <c r="BU14" s="35" t="s">
+      <c r="BT14" s="14" t="s">
+        <v>982</v>
+      </c>
+      <c r="BU14" s="34" t="s">
         <v>179</v>
       </c>
       <c r="BV14" s="7" t="s">
         <v>889</v>
       </c>
-      <c r="BW14" s="13">
+      <c r="BW14" s="12">
         <v>19</v>
       </c>
-      <c r="BX14" s="13">
+      <c r="BX14" s="12">
         <v>1</v>
       </c>
       <c r="BY14" s="7" t="s">
@@ -7876,7 +7853,7 @@
       <c r="CA14" s="11" t="s">
         <v>490</v>
       </c>
-      <c r="CB14" s="13">
+      <c r="CB14" s="12">
         <v>65143</v>
       </c>
       <c r="CC14" s="7" t="s">
@@ -7885,7 +7862,7 @@
       <c r="CD14" s="7" t="s">
         <v>162</v>
       </c>
-      <c r="CE14" s="13" t="s">
+      <c r="CE14" s="12" t="s">
         <v>182</v>
       </c>
       <c r="CF14" s="7" t="s">
@@ -7900,7 +7877,7 @@
       <c r="CI14" s="7" t="s">
         <v>152</v>
       </c>
-      <c r="CJ14" s="13" t="s">
+      <c r="CJ14" s="12" t="s">
         <v>152</v>
       </c>
       <c r="CK14" s="7" t="s">
@@ -7918,7 +7895,7 @@
       <c r="CO14" s="7" t="s">
         <v>152</v>
       </c>
-      <c r="CP14" s="13"/>
+      <c r="CP14" s="12"/>
       <c r="CQ14" s="7" t="s">
         <v>152</v>
       </c>
@@ -7969,10 +7946,10 @@
       </c>
     </row>
     <row r="15" spans="1:113" s="7" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="13">
+      <c r="A15" s="12">
         <v>14</v>
       </c>
-      <c r="B15" s="15" t="s">
+      <c r="B15" s="14" t="s">
         <v>831</v>
       </c>
       <c r="C15" s="7" t="s">
@@ -7982,48 +7959,48 @@
         <v>837</v>
       </c>
       <c r="E15" s="7" t="s">
+        <v>983</v>
+      </c>
+      <c r="F15" s="13" t="s">
+        <v>935</v>
+      </c>
+      <c r="G15" s="13" t="s">
+        <v>814</v>
+      </c>
+      <c r="H15" s="36" t="s">
+        <v>1032</v>
+      </c>
+      <c r="I15" s="13" t="s">
         <v>984</v>
       </c>
-      <c r="F15" s="14" t="s">
-        <v>936</v>
-      </c>
-      <c r="G15" s="14" t="s">
-        <v>814</v>
-      </c>
-      <c r="H15" s="37" t="s">
-        <v>1033</v>
-      </c>
-      <c r="I15" s="14" t="s">
-        <v>985</v>
-      </c>
-      <c r="J15" s="13" t="s">
+      <c r="J15" s="12" t="s">
         <v>704</v>
       </c>
       <c r="K15" s="7" t="s">
         <v>701</v>
       </c>
-      <c r="L15" s="13">
+      <c r="L15" s="12">
         <v>7</v>
       </c>
-      <c r="M15" s="13" t="s">
+      <c r="M15" s="12" t="s">
         <v>801</v>
       </c>
-      <c r="N15" s="13" t="s">
+      <c r="N15" s="12" t="s">
         <v>702</v>
       </c>
-      <c r="O15" s="13" t="s">
+      <c r="O15" s="12" t="s">
         <v>703</v>
       </c>
-      <c r="P15" s="13" t="s">
+      <c r="P15" s="12" t="s">
         <v>286</v>
       </c>
-      <c r="Q15" s="13" t="s">
+      <c r="Q15" s="12" t="s">
         <v>226</v>
       </c>
-      <c r="R15" s="17" t="s">
+      <c r="R15" s="16" t="s">
         <v>767</v>
       </c>
-      <c r="S15" s="17" t="e">
+      <c r="S15" s="16" t="e">
         <f t="shared" ca="1" si="2"/>
         <v>#VALUE!</v>
       </c>
@@ -8033,10 +8010,10 @@
       <c r="V15" s="7" t="s">
         <v>776</v>
       </c>
-      <c r="W15" s="13" t="s">
+      <c r="W15" s="12" t="s">
         <v>577</v>
       </c>
-      <c r="X15" s="13" t="s">
+      <c r="X15" s="12" t="s">
         <v>346</v>
       </c>
       <c r="Y15" s="7" t="s">
@@ -8048,7 +8025,7 @@
       <c r="AA15" s="7" t="s">
         <v>490</v>
       </c>
-      <c r="AB15" s="13">
+      <c r="AB15" s="12">
         <v>65142</v>
       </c>
       <c r="AC15" s="7" t="s">
@@ -8084,13 +8061,13 @@
       <c r="AN15" s="7" t="s">
         <v>236</v>
       </c>
-      <c r="AO15" s="13">
+      <c r="AO15" s="12">
         <v>60</v>
       </c>
-      <c r="AP15" s="13">
+      <c r="AP15" s="12">
         <v>155</v>
       </c>
-      <c r="AQ15" s="13" t="s">
+      <c r="AQ15" s="12" t="s">
         <v>164</v>
       </c>
       <c r="AR15" s="7" t="s">
@@ -8108,8 +8085,8 @@
       <c r="AV15" s="7" t="s">
         <v>711</v>
       </c>
-      <c r="AW15" s="15" t="s">
-        <v>986</v>
+      <c r="AW15" s="14" t="s">
+        <v>985</v>
       </c>
       <c r="AX15" s="7" t="s">
         <v>712</v>
@@ -8117,10 +8094,10 @@
       <c r="AY15" s="7" t="s">
         <v>858</v>
       </c>
-      <c r="BA15" s="13" t="s">
+      <c r="BA15" s="12" t="s">
         <v>577</v>
       </c>
-      <c r="BB15" s="13" t="s">
+      <c r="BB15" s="12" t="s">
         <v>346</v>
       </c>
       <c r="BC15" s="7" t="s">
@@ -8132,16 +8109,16 @@
       <c r="BE15" s="7" t="s">
         <v>490</v>
       </c>
-      <c r="BF15" s="13">
+      <c r="BF15" s="12">
         <v>65142</v>
       </c>
       <c r="BG15" s="7" t="s">
         <v>161</v>
       </c>
-      <c r="BH15" s="13" t="s">
+      <c r="BH15" s="12" t="s">
         <v>162</v>
       </c>
-      <c r="BI15" s="13" t="s">
+      <c r="BI15" s="12" t="s">
         <v>715</v>
       </c>
       <c r="BJ15" s="7" t="s">
@@ -8157,10 +8134,10 @@
       <c r="BM15" s="7" t="s">
         <v>858</v>
       </c>
-      <c r="BN15" s="13" t="s">
+      <c r="BN15" s="12" t="s">
         <v>715</v>
       </c>
-      <c r="BO15" s="21" t="s">
+      <c r="BO15" s="20" t="s">
         <v>718</v>
       </c>
       <c r="BP15" s="7" t="s">
@@ -8175,7 +8152,7 @@
       <c r="BS15" s="7" t="s">
         <v>226</v>
       </c>
-      <c r="BT15" s="15" t="s">
+      <c r="BT15" s="14" t="s">
         <v>152</v>
       </c>
       <c r="BU15" s="7" t="s">
@@ -8184,10 +8161,10 @@
       <c r="BV15" s="7" t="s">
         <v>152</v>
       </c>
-      <c r="BW15" s="13" t="s">
-        <v>152</v>
-      </c>
-      <c r="BX15" s="13" t="s">
+      <c r="BW15" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="BX15" s="12" t="s">
         <v>152</v>
       </c>
       <c r="BY15" s="7" t="s">
@@ -8199,7 +8176,7 @@
       <c r="CA15" s="7" t="s">
         <v>152</v>
       </c>
-      <c r="CB15" s="13" t="s">
+      <c r="CB15" s="12" t="s">
         <v>152</v>
       </c>
       <c r="CC15" s="7" t="s">
@@ -8208,7 +8185,7 @@
       <c r="CD15" s="7" t="s">
         <v>162</v>
       </c>
-      <c r="CE15" s="13" t="s">
+      <c r="CE15" s="12" t="s">
         <v>152</v>
       </c>
       <c r="CF15" s="7" t="s">
@@ -8223,7 +8200,7 @@
       <c r="CI15" s="7" t="s">
         <v>152</v>
       </c>
-      <c r="CJ15" s="13" t="s">
+      <c r="CJ15" s="12" t="s">
         <v>152</v>
       </c>
       <c r="CK15" s="7" t="s">
@@ -8241,7 +8218,7 @@
       <c r="CO15" s="11" t="s">
         <v>226</v>
       </c>
-      <c r="CP15" s="13">
+      <c r="CP15" s="12">
         <v>37481</v>
       </c>
       <c r="CQ15" s="7" t="s">
@@ -8297,18 +8274,16 @@
       </c>
     </row>
     <row r="16" spans="1:113" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B16" s="16"/>
-      <c r="H16" s="16"/>
-      <c r="R16" s="12"/>
-      <c r="S16" s="12"/>
-      <c r="AW16" s="16"/>
-      <c r="BT16" s="16"/>
+      <c r="B16" s="15"/>
+      <c r="H16" s="15"/>
+      <c r="AW16" s="15"/>
+      <c r="BT16" s="15"/>
     </row>
     <row r="17" spans="72:72" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="BT17" s="16"/>
+      <c r="BT17" s="15"/>
     </row>
     <row r="18" spans="72:72" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="BT18" s="16"/>
+      <c r="BT18" s="15"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:DH14" xr:uid="{00000000-0001-0000-0000-000000000000}">

</xml_diff>